<commit_message>
test/Updated Shopping Cart Testcases
</commit_message>
<xml_diff>
--- a/TestCases_Docs/ShoppingCart_TestCases.xlsx
+++ b/TestCases_Docs/ShoppingCart_TestCases.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lenovo\Videos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lenovo\OneDrive\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{786280DF-F4A6-488F-8796-78E863D7288C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{021F7BE5-8290-4F7E-A076-FB55A20AB955}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="11520" windowHeight="12360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cart Test Cases" sheetId="5" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1132" uniqueCount="366">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1132" uniqueCount="367">
   <si>
     <t>TesTCASE ID</t>
   </si>
@@ -266,11 +266,6 @@
   </si>
   <si>
     <t>Verify that clicking the trash icon removes the item from the cart</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 1. Client has a valid account   
-2. Client is logged in  
- 3. Cart contains at least one product</t>
   </si>
   <si>
     <t>1. Add a product to cart 
@@ -1648,6 +1643,16 @@
 5. fill all fields with valid data
 6. return to first user
 7. Navigate to Cart page</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 1. Client has a valid account   
+2. Client is logged in  
+ 3. Cart is empty</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 1. Client has a valid account   
+2. Client is logged in  
+ 3. Cart is Empty</t>
   </si>
 </sst>
 </file>
@@ -1919,7 +1924,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="2"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2067,9 +2072,6 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -2079,6 +2081,137 @@
     <cellStyle name="Normal 2" xfId="1" xr:uid="{6E553DE7-9013-4E7A-B3F3-1617D60456E3}"/>
   </cellStyles>
   <dxfs count="60">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
     <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
@@ -2234,18 +2367,70 @@
       </border>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7"/>
-        </patternFill>
-      </fill>
+      <border>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -2265,47 +2450,14 @@
       </border>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <family val="2"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
       <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
-        <right/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
         <top style="thin">
           <color indexed="64"/>
         </top>
@@ -2383,7 +2535,7 @@
       </border>
     </dxf>
     <dxf>
-      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
@@ -2401,7 +2553,7 @@
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
+      <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -2414,6 +2566,8 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
+        <vertical/>
+        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -2555,13 +2709,6 @@
         <top style="thin">
           <color rgb="FF000000"/>
         </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <bottom style="thin">
-          <color rgb="FF000000"/>
-        </bottom>
       </border>
     </dxf>
     <dxf>
@@ -2584,127 +2731,18 @@
       <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
+      <border>
         <bottom style="thin">
-          <color indexed="64"/>
+          <color rgb="FF000000"/>
         </bottom>
       </border>
     </dxf>
     <dxf>
-      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <font>
+        <b/>
+        <family val="2"/>
+      </font>
       <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -2713,42 +2751,6 @@
         </right>
         <top/>
         <bottom/>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
       </border>
     </dxf>
     <dxf>
@@ -2938,50 +2940,50 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{CA9B46E1-5155-4AAF-844B-BCD9CCA2EDF6}" name="Table17" displayName="Table17" ref="A1:O20" totalsRowShown="0" headerRowDxfId="40" dataDxfId="32" headerRowBorderDxfId="42" tableBorderDxfId="43" totalsRowBorderDxfId="41">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{CA9B46E1-5155-4AAF-844B-BCD9CCA2EDF6}" name="Table17" displayName="Table17" ref="A1:O20" totalsRowShown="0" headerRowDxfId="21" dataDxfId="19" headerRowBorderDxfId="20" tableBorderDxfId="18" totalsRowBorderDxfId="17">
   <autoFilter ref="A1:O20" xr:uid="{CA9B46E1-5155-4AAF-844B-BCD9CCA2EDF6}"/>
   <tableColumns count="15">
-    <tableColumn id="1" xr3:uid="{11F6C013-4C48-4E7A-B8F8-375AECFF097E}" name="TesTCASE ID" dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{1B888F99-A907-40FC-B776-834DD24F6F57}" name="Test Cases Title " dataDxfId="6"/>
-    <tableColumn id="3" xr3:uid="{7853AC75-B7A3-4B9B-B597-0CC90E8D52BF}" name="valid/invalid" dataDxfId="5"/>
-    <tableColumn id="4" xr3:uid="{AAABAF80-25C1-4ACB-ADF4-7337AEA0E0A4}" name="Environment" dataDxfId="4"/>
-    <tableColumn id="5" xr3:uid="{050A3DD3-5C3B-40E3-B68A-DE6E46C20CD3}" name="Pre-condition" dataDxfId="3"/>
-    <tableColumn id="6" xr3:uid="{695FB61F-899E-47FB-AC04-D25E8F4EFFA9}" name="Steps" dataDxfId="2"/>
-    <tableColumn id="7" xr3:uid="{6AADAA49-15BA-4E3C-B63A-DDA3E7EF4C96}" name="Test Data" dataDxfId="1"/>
-    <tableColumn id="8" xr3:uid="{C1CE8F53-60B8-411D-A252-48EAF0B6899D}" name="Expected Results" dataDxfId="0"/>
-    <tableColumn id="9" xr3:uid="{5CBA8F0E-EFB2-441E-ABB2-C8AFC9733678}" name="Post Condition" dataDxfId="39"/>
-    <tableColumn id="10" xr3:uid="{F1F2F7F1-026F-45A0-971C-F5B647193AEB}" name="TC Status" dataDxfId="38"/>
-    <tableColumn id="11" xr3:uid="{C1B2E8E9-0DE1-4E62-B972-DE5006C951AE}" name="Attachment" dataDxfId="37"/>
-    <tableColumn id="12" xr3:uid="{3F1A62C0-FBFC-41F2-B1C9-42BCC073A738}" name="Requirement ID" dataDxfId="36"/>
-    <tableColumn id="13" xr3:uid="{FF0D4754-9DCA-4527-96A7-45E4EA4C6EED}" name="Type" dataDxfId="35"/>
-    <tableColumn id="14" xr3:uid="{CEE95E6B-C591-4C14-8305-FA320F301C59}" name="Tester" dataDxfId="34"/>
-    <tableColumn id="15" xr3:uid="{678D806D-10AD-4D08-AE9F-776FEBFD7C5C}" name="Comment" dataDxfId="33"/>
+    <tableColumn id="1" xr3:uid="{11F6C013-4C48-4E7A-B8F8-375AECFF097E}" name="TesTCASE ID" dataDxfId="16"/>
+    <tableColumn id="2" xr3:uid="{1B888F99-A907-40FC-B776-834DD24F6F57}" name="Test Cases Title " dataDxfId="15"/>
+    <tableColumn id="3" xr3:uid="{7853AC75-B7A3-4B9B-B597-0CC90E8D52BF}" name="valid/invalid" dataDxfId="14"/>
+    <tableColumn id="4" xr3:uid="{AAABAF80-25C1-4ACB-ADF4-7337AEA0E0A4}" name="Environment" dataDxfId="13"/>
+    <tableColumn id="5" xr3:uid="{050A3DD3-5C3B-40E3-B68A-DE6E46C20CD3}" name="Pre-condition" dataDxfId="12"/>
+    <tableColumn id="6" xr3:uid="{695FB61F-899E-47FB-AC04-D25E8F4EFFA9}" name="Steps" dataDxfId="11"/>
+    <tableColumn id="7" xr3:uid="{6AADAA49-15BA-4E3C-B63A-DDA3E7EF4C96}" name="Test Data" dataDxfId="10"/>
+    <tableColumn id="8" xr3:uid="{C1CE8F53-60B8-411D-A252-48EAF0B6899D}" name="Expected Results" dataDxfId="9"/>
+    <tableColumn id="9" xr3:uid="{5CBA8F0E-EFB2-441E-ABB2-C8AFC9733678}" name="Post Condition" dataDxfId="8"/>
+    <tableColumn id="10" xr3:uid="{F1F2F7F1-026F-45A0-971C-F5B647193AEB}" name="TC Status" dataDxfId="7"/>
+    <tableColumn id="11" xr3:uid="{C1B2E8E9-0DE1-4E62-B972-DE5006C951AE}" name="Attachment" dataDxfId="6"/>
+    <tableColumn id="12" xr3:uid="{3F1A62C0-FBFC-41F2-B1C9-42BCC073A738}" name="Requirement ID" dataDxfId="5"/>
+    <tableColumn id="13" xr3:uid="{FF0D4754-9DCA-4527-96A7-45E4EA4C6EED}" name="Type" dataDxfId="4"/>
+    <tableColumn id="14" xr3:uid="{CEE95E6B-C591-4C14-8305-FA320F301C59}" name="Tester" dataDxfId="3"/>
+    <tableColumn id="15" xr3:uid="{678D806D-10AD-4D08-AE9F-776FEBFD7C5C}" name="Comment" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="Cart Test Cases-style" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="18" xr:uid="{7DE26239-599D-4E8A-B29E-9F20DE12A166}" name="Table1719" displayName="Table1719" ref="A1:Q20" totalsRowShown="0" headerRowDxfId="12" dataDxfId="31" headerRowBorderDxfId="29" tableBorderDxfId="30" totalsRowBorderDxfId="28">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="18" xr:uid="{7DE26239-599D-4E8A-B29E-9F20DE12A166}" name="Table1719" displayName="Table1719" ref="A1:Q20" totalsRowShown="0" headerRowDxfId="43" dataDxfId="41" headerRowBorderDxfId="42" tableBorderDxfId="40" totalsRowBorderDxfId="39">
   <autoFilter ref="A1:Q20" xr:uid="{CA9B46E1-5155-4AAF-844B-BCD9CCA2EDF6}"/>
   <tableColumns count="17">
-    <tableColumn id="1" xr3:uid="{6349AC1B-18C1-4513-A98D-74004451BE07}" name="TesTCASE ID" dataDxfId="27"/>
-    <tableColumn id="2" xr3:uid="{316A01E1-D06A-4667-AE3C-453DBC4B1054}" name="Test Cases Title " dataDxfId="26"/>
-    <tableColumn id="3" xr3:uid="{8F7A3C5E-7DAA-4BE5-BB4C-4242660A0347}" name="valid/invalid" dataDxfId="25"/>
-    <tableColumn id="4" xr3:uid="{6F77ADFD-1C3F-4A08-A6E4-478BE3CD7F59}" name="Environment" dataDxfId="24"/>
-    <tableColumn id="5" xr3:uid="{519F839C-1B74-4449-9BE1-EDCA27C25137}" name="Pre-condition" dataDxfId="23"/>
-    <tableColumn id="6" xr3:uid="{F29F0414-7871-4D01-A1DD-A280EE6716F5}" name="Steps" dataDxfId="22"/>
-    <tableColumn id="7" xr3:uid="{2749E69B-C03F-4456-97F1-16E4C7DAB4C8}" name="Test Data" dataDxfId="21"/>
-    <tableColumn id="8" xr3:uid="{10DFC294-FAB0-4D43-8B83-7C0CE4E11BE0}" name="Expected Results" dataDxfId="20"/>
-    <tableColumn id="16" xr3:uid="{2D24DDBD-5A02-4264-B89B-27175D91D43D}" name="Actual result" dataDxfId="11"/>
-    <tableColumn id="9" xr3:uid="{B771E747-8E01-4980-9B14-221C5B00CF89}" name="Post Condition" dataDxfId="19"/>
-    <tableColumn id="10" xr3:uid="{903AF337-308B-4432-90B3-453B150C8696}" name="TC Status" dataDxfId="18"/>
-    <tableColumn id="11" xr3:uid="{DA7982CC-CFB4-46EF-8D7D-498270ACE130}" name="Attachment" dataDxfId="17"/>
-    <tableColumn id="12" xr3:uid="{C3C4BBD3-BE51-4BB4-A9C8-4688454A9D7B}" name="Requirement ID" dataDxfId="16"/>
-    <tableColumn id="13" xr3:uid="{6FFDB195-604A-4141-B2B3-FB2EBCCF9EE1}" name="Type" dataDxfId="15"/>
-    <tableColumn id="14" xr3:uid="{0C076CE8-316D-4323-B69F-E0CA15A82960}" name="Tester" dataDxfId="14"/>
-    <tableColumn id="17" xr3:uid="{C124139E-C07E-4913-834E-C22FF51CDDC5}" name="Execution_Status" dataDxfId="10"/>
-    <tableColumn id="15" xr3:uid="{7B9BAC1F-276D-47AE-B4F7-FBBDF0CA5C1C}" name="Comment" dataDxfId="13"/>
+    <tableColumn id="1" xr3:uid="{6349AC1B-18C1-4513-A98D-74004451BE07}" name="TesTCASE ID" dataDxfId="38"/>
+    <tableColumn id="2" xr3:uid="{316A01E1-D06A-4667-AE3C-453DBC4B1054}" name="Test Cases Title " dataDxfId="37"/>
+    <tableColumn id="3" xr3:uid="{8F7A3C5E-7DAA-4BE5-BB4C-4242660A0347}" name="valid/invalid" dataDxfId="36"/>
+    <tableColumn id="4" xr3:uid="{6F77ADFD-1C3F-4A08-A6E4-478BE3CD7F59}" name="Environment" dataDxfId="35"/>
+    <tableColumn id="5" xr3:uid="{519F839C-1B74-4449-9BE1-EDCA27C25137}" name="Pre-condition" dataDxfId="34"/>
+    <tableColumn id="6" xr3:uid="{F29F0414-7871-4D01-A1DD-A280EE6716F5}" name="Steps" dataDxfId="33"/>
+    <tableColumn id="7" xr3:uid="{2749E69B-C03F-4456-97F1-16E4C7DAB4C8}" name="Test Data" dataDxfId="32"/>
+    <tableColumn id="8" xr3:uid="{10DFC294-FAB0-4D43-8B83-7C0CE4E11BE0}" name="Expected Results" dataDxfId="31"/>
+    <tableColumn id="16" xr3:uid="{2D24DDBD-5A02-4264-B89B-27175D91D43D}" name="Actual result" dataDxfId="30"/>
+    <tableColumn id="9" xr3:uid="{B771E747-8E01-4980-9B14-221C5B00CF89}" name="Post Condition" dataDxfId="29"/>
+    <tableColumn id="10" xr3:uid="{903AF337-308B-4432-90B3-453B150C8696}" name="TC Status" dataDxfId="28"/>
+    <tableColumn id="11" xr3:uid="{DA7982CC-CFB4-46EF-8D7D-498270ACE130}" name="Attachment" dataDxfId="27"/>
+    <tableColumn id="12" xr3:uid="{C3C4BBD3-BE51-4BB4-A9C8-4688454A9D7B}" name="Requirement ID" dataDxfId="26"/>
+    <tableColumn id="13" xr3:uid="{6FFDB195-604A-4141-B2B3-FB2EBCCF9EE1}" name="Type" dataDxfId="25"/>
+    <tableColumn id="14" xr3:uid="{0C076CE8-316D-4323-B69F-E0CA15A82960}" name="Tester" dataDxfId="24"/>
+    <tableColumn id="17" xr3:uid="{C124139E-C07E-4913-834E-C22FF51CDDC5}" name="Execution_Status" dataDxfId="23"/>
+    <tableColumn id="15" xr3:uid="{7B9BAC1F-276D-47AE-B4F7-FBBDF0CA5C1C}" name="Comment" dataDxfId="22"/>
   </tableColumns>
   <tableStyleInfo name="Cart Test Cases-style" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3272,7 +3274,7 @@
         <v>20</v>
       </c>
       <c r="G2" s="53" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="H2" s="42" t="s">
         <v>21</v>
@@ -3317,7 +3319,7 @@
         <v>29</v>
       </c>
       <c r="G3" s="53" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="H3" s="42" t="s">
         <v>30</v>
@@ -3362,7 +3364,7 @@
         <v>33</v>
       </c>
       <c r="G4" s="53" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="H4" s="42" t="s">
         <v>34</v>
@@ -3407,7 +3409,7 @@
         <v>38</v>
       </c>
       <c r="G5" s="53" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="H5" s="42" t="s">
         <v>39</v>
@@ -3452,7 +3454,7 @@
         <v>42</v>
       </c>
       <c r="G6" s="53" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="H6" s="42" t="s">
         <v>43</v>
@@ -3491,13 +3493,13 @@
         <v>18</v>
       </c>
       <c r="E7" s="48" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="F7" s="40" t="s">
         <v>47</v>
       </c>
       <c r="G7" s="53" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="H7" s="42" t="s">
         <v>48</v>
@@ -3536,13 +3538,13 @@
         <v>18</v>
       </c>
       <c r="E8" s="48" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="F8" s="40" t="s">
         <v>51</v>
       </c>
       <c r="G8" s="53" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="H8" s="42" t="s">
         <v>52</v>
@@ -3581,13 +3583,13 @@
         <v>18</v>
       </c>
       <c r="E9" s="48" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="F9" s="40" t="s">
         <v>55</v>
       </c>
       <c r="G9" s="53" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="H9" s="42" t="s">
         <v>56</v>
@@ -3632,7 +3634,7 @@
         <v>61</v>
       </c>
       <c r="G10" s="53" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="H10" s="42" t="s">
         <v>62</v>
@@ -3677,7 +3679,7 @@
         <v>66</v>
       </c>
       <c r="G11" s="53" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="H11" s="42" t="s">
         <v>67</v>
@@ -3716,16 +3718,16 @@
         <v>18</v>
       </c>
       <c r="E12" s="42" t="s">
+        <v>366</v>
+      </c>
+      <c r="F12" s="40" t="s">
         <v>70</v>
       </c>
-      <c r="F12" s="40" t="s">
+      <c r="G12" s="53" t="s">
+        <v>351</v>
+      </c>
+      <c r="H12" s="42" t="s">
         <v>71</v>
-      </c>
-      <c r="G12" s="53" t="s">
-        <v>352</v>
-      </c>
-      <c r="H12" s="42" t="s">
-        <v>72</v>
       </c>
       <c r="I12" s="42"/>
       <c r="J12" s="38" t="s">
@@ -3735,7 +3737,7 @@
         <v>23</v>
       </c>
       <c r="L12" s="38" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="M12" s="38" t="s">
         <v>44</v>
@@ -3744,15 +3746,15 @@
         <v>26</v>
       </c>
       <c r="O12" s="43" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="13" spans="1:15" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A13" s="41" t="s">
+        <v>74</v>
+      </c>
+      <c r="B13" s="38" t="s">
         <v>75</v>
-      </c>
-      <c r="B13" s="38" t="s">
-        <v>76</v>
       </c>
       <c r="C13" s="46" t="s">
         <v>17</v>
@@ -3761,16 +3763,16 @@
         <v>18</v>
       </c>
       <c r="E13" s="42" t="s">
+        <v>76</v>
+      </c>
+      <c r="F13" s="40" t="s">
         <v>77</v>
       </c>
-      <c r="F13" s="40" t="s">
+      <c r="G13" s="53" t="s">
+        <v>351</v>
+      </c>
+      <c r="H13" s="42" t="s">
         <v>78</v>
-      </c>
-      <c r="G13" s="53" t="s">
-        <v>352</v>
-      </c>
-      <c r="H13" s="42" t="s">
-        <v>79</v>
       </c>
       <c r="I13" s="42"/>
       <c r="J13" s="38" t="s">
@@ -3780,7 +3782,7 @@
         <v>23</v>
       </c>
       <c r="L13" s="38" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="M13" s="38" t="s">
         <v>44</v>
@@ -3794,10 +3796,10 @@
     </row>
     <row r="14" spans="1:15" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A14" s="41" t="s">
+        <v>79</v>
+      </c>
+      <c r="B14" s="38" t="s">
         <v>80</v>
-      </c>
-      <c r="B14" s="38" t="s">
-        <v>81</v>
       </c>
       <c r="C14" s="46" t="s">
         <v>17</v>
@@ -3806,16 +3808,16 @@
         <v>18</v>
       </c>
       <c r="E14" s="42" t="s">
+        <v>81</v>
+      </c>
+      <c r="F14" s="40" t="s">
         <v>82</v>
       </c>
-      <c r="F14" s="40" t="s">
+      <c r="G14" s="53" t="s">
+        <v>351</v>
+      </c>
+      <c r="H14" s="42" t="s">
         <v>83</v>
-      </c>
-      <c r="G14" s="53" t="s">
-        <v>352</v>
-      </c>
-      <c r="H14" s="42" t="s">
-        <v>84</v>
       </c>
       <c r="I14" s="42"/>
       <c r="J14" s="38" t="s">
@@ -3825,7 +3827,7 @@
         <v>23</v>
       </c>
       <c r="L14" s="38" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="M14" s="38" t="s">
         <v>44</v>
@@ -3839,10 +3841,10 @@
     </row>
     <row r="15" spans="1:15" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A15" s="41" t="s">
+        <v>85</v>
+      </c>
+      <c r="B15" s="38" t="s">
         <v>86</v>
-      </c>
-      <c r="B15" s="38" t="s">
-        <v>87</v>
       </c>
       <c r="C15" s="46" t="s">
         <v>17</v>
@@ -3851,16 +3853,16 @@
         <v>18</v>
       </c>
       <c r="E15" s="42" t="s">
+        <v>87</v>
+      </c>
+      <c r="F15" s="40" t="s">
         <v>88</v>
       </c>
-      <c r="F15" s="40" t="s">
+      <c r="G15" s="53" t="s">
+        <v>351</v>
+      </c>
+      <c r="H15" s="42" t="s">
         <v>89</v>
-      </c>
-      <c r="G15" s="53" t="s">
-        <v>352</v>
-      </c>
-      <c r="H15" s="42" t="s">
-        <v>90</v>
       </c>
       <c r="I15" s="42"/>
       <c r="J15" s="38" t="s">
@@ -3870,7 +3872,7 @@
         <v>23</v>
       </c>
       <c r="L15" s="38" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="M15" s="38" t="s">
         <v>44</v>
@@ -3884,10 +3886,10 @@
     </row>
     <row r="16" spans="1:15" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A16" s="41" t="s">
+        <v>90</v>
+      </c>
+      <c r="B16" s="38" t="s">
         <v>91</v>
-      </c>
-      <c r="B16" s="38" t="s">
-        <v>92</v>
       </c>
       <c r="C16" s="46" t="s">
         <v>17</v>
@@ -3896,16 +3898,16 @@
         <v>18</v>
       </c>
       <c r="E16" s="42" t="s">
+        <v>92</v>
+      </c>
+      <c r="F16" s="40" t="s">
         <v>93</v>
       </c>
-      <c r="F16" s="40" t="s">
+      <c r="G16" s="53" t="s">
+        <v>351</v>
+      </c>
+      <c r="H16" s="42" t="s">
         <v>94</v>
-      </c>
-      <c r="G16" s="53" t="s">
-        <v>352</v>
-      </c>
-      <c r="H16" s="42" t="s">
-        <v>95</v>
       </c>
       <c r="I16" s="42"/>
       <c r="J16" s="38" t="s">
@@ -3915,7 +3917,7 @@
         <v>23</v>
       </c>
       <c r="L16" s="38" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="M16" s="38" t="s">
         <v>44</v>
@@ -3929,10 +3931,10 @@
     </row>
     <row r="17" spans="1:15" ht="52.8" x14ac:dyDescent="0.25">
       <c r="A17" s="41" t="s">
+        <v>95</v>
+      </c>
+      <c r="B17" s="38" t="s">
         <v>96</v>
-      </c>
-      <c r="B17" s="38" t="s">
-        <v>97</v>
       </c>
       <c r="C17" s="46" t="s">
         <v>17</v>
@@ -3941,16 +3943,16 @@
         <v>18</v>
       </c>
       <c r="E17" s="42" t="s">
+        <v>97</v>
+      </c>
+      <c r="F17" s="40" t="s">
         <v>98</v>
       </c>
-      <c r="F17" s="40" t="s">
+      <c r="G17" s="53" t="s">
+        <v>351</v>
+      </c>
+      <c r="H17" s="42" t="s">
         <v>99</v>
-      </c>
-      <c r="G17" s="53" t="s">
-        <v>352</v>
-      </c>
-      <c r="H17" s="42" t="s">
-        <v>100</v>
       </c>
       <c r="I17" s="42"/>
       <c r="J17" s="38" t="s">
@@ -3960,13 +3962,13 @@
         <v>23</v>
       </c>
       <c r="L17" s="38" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="M17" s="38" t="s">
         <v>44</v>
       </c>
       <c r="N17" s="38" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="O17" s="43" t="s">
         <v>23</v>
@@ -3974,10 +3976,10 @@
     </row>
     <row r="18" spans="1:15" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A18" s="41" t="s">
+        <v>101</v>
+      </c>
+      <c r="B18" s="38" t="s">
         <v>102</v>
-      </c>
-      <c r="B18" s="38" t="s">
-        <v>103</v>
       </c>
       <c r="C18" s="46" t="s">
         <v>17</v>
@@ -3986,16 +3988,16 @@
         <v>18</v>
       </c>
       <c r="E18" s="42" t="s">
+        <v>103</v>
+      </c>
+      <c r="F18" s="40" t="s">
         <v>104</v>
       </c>
-      <c r="F18" s="40" t="s">
+      <c r="G18" s="53" t="s">
+        <v>351</v>
+      </c>
+      <c r="H18" s="42" t="s">
         <v>105</v>
-      </c>
-      <c r="G18" s="53" t="s">
-        <v>352</v>
-      </c>
-      <c r="H18" s="42" t="s">
-        <v>106</v>
       </c>
       <c r="I18" s="42"/>
       <c r="J18" s="38" t="s">
@@ -4005,13 +4007,13 @@
         <v>23</v>
       </c>
       <c r="L18" s="38" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="M18" s="38" t="s">
         <v>25</v>
       </c>
       <c r="N18" s="38" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="O18" s="43" t="s">
         <v>23</v>
@@ -4019,28 +4021,28 @@
     </row>
     <row r="19" spans="1:15" ht="92.4" x14ac:dyDescent="0.25">
       <c r="A19" s="41" t="s">
+        <v>106</v>
+      </c>
+      <c r="B19" s="38" t="s">
+        <v>109</v>
+      </c>
+      <c r="C19" s="46" t="s">
         <v>107</v>
-      </c>
-      <c r="B19" s="38" t="s">
-        <v>110</v>
-      </c>
-      <c r="C19" s="46" t="s">
-        <v>108</v>
       </c>
       <c r="D19" s="46" t="s">
         <v>18</v>
       </c>
       <c r="E19" s="42" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F19" s="54" t="s">
+        <v>362</v>
+      </c>
+      <c r="G19" s="53" t="s">
         <v>363</v>
       </c>
-      <c r="G19" s="53" t="s">
-        <v>364</v>
-      </c>
       <c r="H19" s="48" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="I19" s="42"/>
       <c r="J19" s="38" t="s">
@@ -4049,14 +4051,14 @@
       <c r="K19" s="38" t="s">
         <v>23</v>
       </c>
-      <c r="L19" s="58" t="s">
-        <v>359</v>
+      <c r="L19" s="57" t="s">
+        <v>358</v>
       </c>
       <c r="M19" s="38" t="s">
         <v>44</v>
       </c>
       <c r="N19" s="38" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="O19" s="43" t="s">
         <v>23</v>
@@ -4064,28 +4066,28 @@
     </row>
     <row r="20" spans="1:15" ht="92.4" x14ac:dyDescent="0.25">
       <c r="A20" s="41" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B20" s="39" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C20" s="47" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D20" s="47" t="s">
         <v>18</v>
       </c>
       <c r="E20" s="55" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="F20" s="56" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="G20" s="53" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="H20" s="55" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="I20" s="44"/>
       <c r="J20" s="39" t="s">
@@ -4094,14 +4096,14 @@
       <c r="K20" s="39" t="s">
         <v>23</v>
       </c>
-      <c r="L20" s="58" t="s">
-        <v>359</v>
+      <c r="L20" s="57" t="s">
+        <v>358</v>
       </c>
       <c r="M20" s="39" t="s">
         <v>44</v>
       </c>
       <c r="N20" s="39" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="O20" s="45" t="s">
         <v>23</v>
@@ -4168,7 +4170,7 @@
         <v>7</v>
       </c>
       <c r="I1" s="50" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="J1" s="50" t="s">
         <v>8</v>
@@ -4189,7 +4191,7 @@
         <v>13</v>
       </c>
       <c r="P1" s="51" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="Q1" s="51" t="s">
         <v>14</v>
@@ -4215,7 +4217,7 @@
         <v>20</v>
       </c>
       <c r="G2" s="53" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="H2" s="42" t="s">
         <v>21</v>
@@ -4240,7 +4242,7 @@
         <v>26</v>
       </c>
       <c r="P2" s="52" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="Q2" s="43" t="s">
         <v>23</v>
@@ -4266,7 +4268,7 @@
         <v>29</v>
       </c>
       <c r="G3" s="53" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="H3" s="42" t="s">
         <v>30</v>
@@ -4291,7 +4293,7 @@
         <v>26</v>
       </c>
       <c r="P3" s="52" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="Q3" s="43" t="s">
         <v>23</v>
@@ -4317,7 +4319,7 @@
         <v>33</v>
       </c>
       <c r="G4" s="53" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="H4" s="42" t="s">
         <v>34</v>
@@ -4342,7 +4344,7 @@
         <v>26</v>
       </c>
       <c r="P4" s="52" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="Q4" s="43" t="s">
         <v>23</v>
@@ -4368,7 +4370,7 @@
         <v>38</v>
       </c>
       <c r="G5" s="53" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="H5" s="42" t="s">
         <v>39</v>
@@ -4393,7 +4395,7 @@
         <v>26</v>
       </c>
       <c r="P5" s="52" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="Q5" s="43" t="s">
         <v>23</v>
@@ -4419,7 +4421,7 @@
         <v>42</v>
       </c>
       <c r="G6" s="53" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="H6" s="42" t="s">
         <v>43</v>
@@ -4444,7 +4446,7 @@
         <v>26</v>
       </c>
       <c r="P6" s="52" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="Q6" s="43" t="s">
         <v>23</v>
@@ -4464,19 +4466,19 @@
         <v>18</v>
       </c>
       <c r="E7" s="48" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="F7" s="40" t="s">
         <v>47</v>
       </c>
       <c r="G7" s="53" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="H7" s="42" t="s">
         <v>48</v>
       </c>
       <c r="I7" s="48" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="J7" s="42"/>
       <c r="K7" s="38" t="s">
@@ -4495,7 +4497,7 @@
         <v>26</v>
       </c>
       <c r="P7" s="52" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="Q7" s="43" t="s">
         <v>23</v>
@@ -4515,13 +4517,13 @@
         <v>18</v>
       </c>
       <c r="E8" s="48" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="F8" s="40" t="s">
         <v>51</v>
       </c>
       <c r="G8" s="53" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="H8" s="42" t="s">
         <v>52</v>
@@ -4546,7 +4548,7 @@
         <v>26</v>
       </c>
       <c r="P8" s="52" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="Q8" s="43" t="s">
         <v>23</v>
@@ -4566,13 +4568,13 @@
         <v>18</v>
       </c>
       <c r="E9" s="48" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="F9" s="40" t="s">
         <v>55</v>
       </c>
       <c r="G9" s="53" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="H9" s="42" t="s">
         <v>56</v>
@@ -4597,7 +4599,7 @@
         <v>26</v>
       </c>
       <c r="P9" s="52" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="Q9" s="43" t="s">
         <v>23</v>
@@ -4623,7 +4625,7 @@
         <v>61</v>
       </c>
       <c r="G10" s="53" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="H10" s="42" t="s">
         <v>62</v>
@@ -4648,7 +4650,7 @@
         <v>26</v>
       </c>
       <c r="P10" s="52" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="Q10" s="43" t="s">
         <v>23</v>
@@ -4674,13 +4676,13 @@
         <v>66</v>
       </c>
       <c r="G11" s="53" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="H11" s="42" t="s">
         <v>67</v>
       </c>
       <c r="I11" s="48" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="J11" s="42"/>
       <c r="K11" s="38" t="s">
@@ -4699,7 +4701,7 @@
         <v>26</v>
       </c>
       <c r="P11" s="52" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="Q11" s="43" t="s">
         <v>23</v>
@@ -4719,19 +4721,19 @@
         <v>18</v>
       </c>
       <c r="E12" s="42" t="s">
+        <v>365</v>
+      </c>
+      <c r="F12" s="40" t="s">
         <v>70</v>
       </c>
-      <c r="F12" s="40" t="s">
+      <c r="G12" s="53" t="s">
+        <v>351</v>
+      </c>
+      <c r="H12" s="42" t="s">
         <v>71</v>
       </c>
-      <c r="G12" s="53" t="s">
-        <v>352</v>
-      </c>
-      <c r="H12" s="42" t="s">
-        <v>72</v>
-      </c>
       <c r="I12" s="48" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="J12" s="42"/>
       <c r="K12" s="38" t="s">
@@ -4741,7 +4743,7 @@
         <v>23</v>
       </c>
       <c r="M12" s="38" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="N12" s="38" t="s">
         <v>44</v>
@@ -4750,18 +4752,18 @@
         <v>26</v>
       </c>
       <c r="P12" s="52" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="Q12" s="43" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="13" spans="1:17" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A13" s="41" t="s">
+        <v>74</v>
+      </c>
+      <c r="B13" s="38" t="s">
         <v>75</v>
-      </c>
-      <c r="B13" s="38" t="s">
-        <v>76</v>
       </c>
       <c r="C13" s="46" t="s">
         <v>17</v>
@@ -4770,19 +4772,19 @@
         <v>18</v>
       </c>
       <c r="E13" s="42" t="s">
+        <v>76</v>
+      </c>
+      <c r="F13" s="40" t="s">
         <v>77</v>
       </c>
-      <c r="F13" s="40" t="s">
+      <c r="G13" s="53" t="s">
+        <v>351</v>
+      </c>
+      <c r="H13" s="42" t="s">
         <v>78</v>
       </c>
-      <c r="G13" s="53" t="s">
-        <v>352</v>
-      </c>
-      <c r="H13" s="42" t="s">
-        <v>79</v>
-      </c>
       <c r="I13" s="42" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="J13" s="42"/>
       <c r="K13" s="38" t="s">
@@ -4792,7 +4794,7 @@
         <v>23</v>
       </c>
       <c r="M13" s="38" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="N13" s="38" t="s">
         <v>44</v>
@@ -4801,7 +4803,7 @@
         <v>26</v>
       </c>
       <c r="P13" s="52" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="Q13" s="43" t="s">
         <v>23</v>
@@ -4809,10 +4811,10 @@
     </row>
     <row r="14" spans="1:17" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A14" s="41" t="s">
+        <v>79</v>
+      </c>
+      <c r="B14" s="38" t="s">
         <v>80</v>
-      </c>
-      <c r="B14" s="38" t="s">
-        <v>81</v>
       </c>
       <c r="C14" s="46" t="s">
         <v>17</v>
@@ -4821,19 +4823,19 @@
         <v>18</v>
       </c>
       <c r="E14" s="42" t="s">
+        <v>81</v>
+      </c>
+      <c r="F14" s="40" t="s">
         <v>82</v>
       </c>
-      <c r="F14" s="40" t="s">
+      <c r="G14" s="53" t="s">
+        <v>351</v>
+      </c>
+      <c r="H14" s="42" t="s">
         <v>83</v>
       </c>
-      <c r="G14" s="53" t="s">
-        <v>352</v>
-      </c>
-      <c r="H14" s="42" t="s">
-        <v>84</v>
-      </c>
       <c r="I14" s="42" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J14" s="42"/>
       <c r="K14" s="38" t="s">
@@ -4843,7 +4845,7 @@
         <v>23</v>
       </c>
       <c r="M14" s="38" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="N14" s="38" t="s">
         <v>44</v>
@@ -4852,7 +4854,7 @@
         <v>26</v>
       </c>
       <c r="P14" s="52" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="Q14" s="43" t="s">
         <v>23</v>
@@ -4860,10 +4862,10 @@
     </row>
     <row r="15" spans="1:17" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A15" s="41" t="s">
+        <v>85</v>
+      </c>
+      <c r="B15" s="38" t="s">
         <v>86</v>
-      </c>
-      <c r="B15" s="38" t="s">
-        <v>87</v>
       </c>
       <c r="C15" s="46" t="s">
         <v>17</v>
@@ -4872,19 +4874,19 @@
         <v>18</v>
       </c>
       <c r="E15" s="42" t="s">
+        <v>87</v>
+      </c>
+      <c r="F15" s="40" t="s">
         <v>88</v>
       </c>
-      <c r="F15" s="40" t="s">
+      <c r="G15" s="53" t="s">
+        <v>351</v>
+      </c>
+      <c r="H15" s="42" t="s">
         <v>89</v>
       </c>
-      <c r="G15" s="53" t="s">
-        <v>352</v>
-      </c>
-      <c r="H15" s="42" t="s">
-        <v>90</v>
-      </c>
       <c r="I15" s="48" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="J15" s="42"/>
       <c r="K15" s="38" t="s">
@@ -4894,7 +4896,7 @@
         <v>23</v>
       </c>
       <c r="M15" s="38" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="N15" s="38" t="s">
         <v>44</v>
@@ -4903,7 +4905,7 @@
         <v>26</v>
       </c>
       <c r="P15" s="52" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="Q15" s="43" t="s">
         <v>23</v>
@@ -4911,10 +4913,10 @@
     </row>
     <row r="16" spans="1:17" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A16" s="41" t="s">
+        <v>90</v>
+      </c>
+      <c r="B16" s="38" t="s">
         <v>91</v>
-      </c>
-      <c r="B16" s="38" t="s">
-        <v>92</v>
       </c>
       <c r="C16" s="46" t="s">
         <v>17</v>
@@ -4923,19 +4925,19 @@
         <v>18</v>
       </c>
       <c r="E16" s="42" t="s">
+        <v>92</v>
+      </c>
+      <c r="F16" s="40" t="s">
         <v>93</v>
       </c>
-      <c r="F16" s="40" t="s">
+      <c r="G16" s="53" t="s">
+        <v>351</v>
+      </c>
+      <c r="H16" s="42" t="s">
         <v>94</v>
       </c>
-      <c r="G16" s="53" t="s">
-        <v>352</v>
-      </c>
-      <c r="H16" s="42" t="s">
-        <v>95</v>
-      </c>
       <c r="I16" s="42" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="J16" s="42"/>
       <c r="K16" s="38" t="s">
@@ -4945,7 +4947,7 @@
         <v>23</v>
       </c>
       <c r="M16" s="38" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="N16" s="38" t="s">
         <v>44</v>
@@ -4954,7 +4956,7 @@
         <v>26</v>
       </c>
       <c r="P16" s="52" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="Q16" s="43" t="s">
         <v>23</v>
@@ -4962,10 +4964,10 @@
     </row>
     <row r="17" spans="1:17" ht="52.8" x14ac:dyDescent="0.25">
       <c r="A17" s="41" t="s">
+        <v>95</v>
+      </c>
+      <c r="B17" s="38" t="s">
         <v>96</v>
-      </c>
-      <c r="B17" s="38" t="s">
-        <v>97</v>
       </c>
       <c r="C17" s="46" t="s">
         <v>17</v>
@@ -4974,19 +4976,19 @@
         <v>18</v>
       </c>
       <c r="E17" s="42" t="s">
+        <v>97</v>
+      </c>
+      <c r="F17" s="40" t="s">
         <v>98</v>
       </c>
-      <c r="F17" s="40" t="s">
+      <c r="G17" s="53" t="s">
+        <v>351</v>
+      </c>
+      <c r="H17" s="42" t="s">
         <v>99</v>
       </c>
-      <c r="G17" s="53" t="s">
-        <v>352</v>
-      </c>
-      <c r="H17" s="42" t="s">
-        <v>100</v>
-      </c>
       <c r="I17" s="42" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="J17" s="42"/>
       <c r="K17" s="38" t="s">
@@ -4996,16 +4998,16 @@
         <v>23</v>
       </c>
       <c r="M17" s="38" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="N17" s="38" t="s">
         <v>44</v>
       </c>
       <c r="O17" s="38" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="P17" s="52" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="Q17" s="43" t="s">
         <v>23</v>
@@ -5013,10 +5015,10 @@
     </row>
     <row r="18" spans="1:17" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A18" s="41" t="s">
+        <v>101</v>
+      </c>
+      <c r="B18" s="38" t="s">
         <v>102</v>
-      </c>
-      <c r="B18" s="38" t="s">
-        <v>103</v>
       </c>
       <c r="C18" s="46" t="s">
         <v>17</v>
@@ -5025,19 +5027,19 @@
         <v>18</v>
       </c>
       <c r="E18" s="42" t="s">
+        <v>103</v>
+      </c>
+      <c r="F18" s="40" t="s">
         <v>104</v>
       </c>
-      <c r="F18" s="40" t="s">
+      <c r="G18" s="53" t="s">
+        <v>351</v>
+      </c>
+      <c r="H18" s="42" t="s">
         <v>105</v>
       </c>
-      <c r="G18" s="53" t="s">
-        <v>352</v>
-      </c>
-      <c r="H18" s="42" t="s">
-        <v>106</v>
-      </c>
       <c r="I18" s="42" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="J18" s="42"/>
       <c r="K18" s="38" t="s">
@@ -5047,16 +5049,16 @@
         <v>23</v>
       </c>
       <c r="M18" s="38" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="N18" s="38" t="s">
         <v>25</v>
       </c>
       <c r="O18" s="38" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="P18" s="52" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="Q18" s="43" t="s">
         <v>23</v>
@@ -5064,31 +5066,31 @@
     </row>
     <row r="19" spans="1:17" ht="92.4" x14ac:dyDescent="0.25">
       <c r="A19" s="41" t="s">
+        <v>106</v>
+      </c>
+      <c r="B19" s="38" t="s">
+        <v>109</v>
+      </c>
+      <c r="C19" s="46" t="s">
         <v>107</v>
-      </c>
-      <c r="B19" s="38" t="s">
-        <v>110</v>
-      </c>
-      <c r="C19" s="46" t="s">
-        <v>108</v>
       </c>
       <c r="D19" s="46" t="s">
         <v>18</v>
       </c>
       <c r="E19" s="42" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F19" s="54" t="s">
+        <v>362</v>
+      </c>
+      <c r="G19" s="53" t="s">
         <v>363</v>
       </c>
-      <c r="G19" s="53" t="s">
-        <v>364</v>
-      </c>
       <c r="H19" s="48" t="s">
+        <v>359</v>
+      </c>
+      <c r="I19" s="48" t="s">
         <v>360</v>
-      </c>
-      <c r="I19" s="48" t="s">
-        <v>361</v>
       </c>
       <c r="J19" s="42"/>
       <c r="K19" s="38" t="s">
@@ -5098,16 +5100,16 @@
         <v>23</v>
       </c>
       <c r="M19" s="57" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="N19" s="38" t="s">
         <v>44</v>
       </c>
       <c r="O19" s="38" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="P19" s="52" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="Q19" s="43" t="s">
         <v>23</v>
@@ -5115,31 +5117,31 @@
     </row>
     <row r="20" spans="1:17" ht="92.4" x14ac:dyDescent="0.25">
       <c r="A20" s="41" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B20" s="39" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C20" s="47" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D20" s="47" t="s">
         <v>18</v>
       </c>
       <c r="E20" s="55" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="F20" s="56" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="G20" s="53" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="H20" s="55" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="I20" s="55" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="J20" s="44"/>
       <c r="K20" s="39" t="s">
@@ -5149,16 +5151,16 @@
         <v>23</v>
       </c>
       <c r="M20" s="57" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="N20" s="39" t="s">
         <v>44</v>
       </c>
       <c r="O20" s="39" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="P20" s="52" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="Q20" s="45" t="s">
         <v>23</v>
@@ -5171,10 +5173,10 @@
   </sheetData>
   <phoneticPr fontId="16" type="noConversion"/>
   <conditionalFormatting sqref="P2:P20">
-    <cfRule type="containsText" dxfId="9" priority="1" operator="containsText" text="Failed">
+    <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="Failed">
       <formula>NOT(ISERROR(SEARCH("Failed",P2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="8" priority="2" operator="containsText" text="Passed">
+    <cfRule type="containsText" dxfId="0" priority="2" operator="containsText" text="Passed">
       <formula>NOT(ISERROR(SEARCH("Passed",P2)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5220,10 +5222,10 @@
         <v>1</v>
       </c>
       <c r="C1" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="D1" s="5" t="s">
         <v>113</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>114</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>4</v>
@@ -5238,7 +5240,7 @@
         <v>7</v>
       </c>
       <c r="I1" s="6" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="J1" s="5" t="s">
         <v>8</v>
@@ -5262,54 +5264,54 @@
         <v>14</v>
       </c>
       <c r="Q1" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="2" spans="1:29" ht="99" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="B2" s="7" t="s">
         <v>117</v>
-      </c>
-      <c r="B2" s="7" t="s">
-        <v>118</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>17</v>
       </c>
       <c r="D2" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="E2" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="F2" s="7" t="s">
         <v>120</v>
       </c>
-      <c r="F2" s="7" t="s">
+      <c r="G2" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="G2" s="7" t="s">
+      <c r="H2" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" s="7" t="s">
         <v>123</v>
-      </c>
-      <c r="I2" s="7" t="s">
-        <v>124</v>
       </c>
       <c r="J2" s="1"/>
       <c r="K2" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="L2" s="1"/>
       <c r="M2" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="N2" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="N2" s="1" t="s">
+      <c r="O2" s="1" t="s">
         <v>127</v>
-      </c>
-      <c r="O2" s="1" t="s">
-        <v>128</v>
       </c>
       <c r="P2" s="1"/>
       <c r="Q2" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="R2" s="1"/>
       <c r="S2" s="1"/>
@@ -5326,49 +5328,49 @@
     </row>
     <row r="3" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="B3" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="C3" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="E3" s="8" t="s">
         <v>131</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="E3" s="8" t="s">
+      <c r="F3" s="7" t="s">
         <v>132</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="G3" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="H3" s="7" t="s">
         <v>134</v>
       </c>
-      <c r="H3" s="7" t="s">
-        <v>135</v>
-      </c>
       <c r="I3" s="7" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="J3" s="1"/>
       <c r="K3" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="L3" s="1"/>
       <c r="M3" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="N3" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="N3" s="1" t="s">
-        <v>127</v>
-      </c>
       <c r="O3" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="P3" s="1"/>
       <c r="Q3" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="R3" s="1"/>
       <c r="S3" s="1"/>
@@ -5385,49 +5387,49 @@
     </row>
     <row r="4" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="B4" s="7" t="s">
         <v>137</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="C4" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="E4" s="8" t="s">
         <v>138</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="E4" s="8" t="s">
+      <c r="F4" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="G4" s="7" t="s">
         <v>139</v>
       </c>
-      <c r="F4" s="7" t="s">
-        <v>133</v>
-      </c>
-      <c r="G4" s="7" t="s">
-        <v>140</v>
-      </c>
       <c r="H4" s="7" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="I4" s="7" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="J4" s="1"/>
       <c r="K4" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="L4" s="1"/>
       <c r="M4" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="N4" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="N4" s="1" t="s">
-        <v>127</v>
-      </c>
       <c r="O4" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="P4" s="1"/>
       <c r="Q4" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="R4" s="1"/>
       <c r="S4" s="1"/>
@@ -5444,49 +5446,49 @@
     </row>
     <row r="5" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="B5" s="7" t="s">
         <v>141</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="C5" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="E5" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="C5" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="E5" s="8" t="s">
+      <c r="F5" s="7" t="s">
         <v>143</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="G5" s="7" t="s">
         <v>144</v>
       </c>
-      <c r="G5" s="7" t="s">
+      <c r="H5" s="7" t="s">
         <v>145</v>
       </c>
-      <c r="H5" s="7" t="s">
-        <v>146</v>
-      </c>
       <c r="I5" s="7" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="J5" s="1"/>
       <c r="K5" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="L5" s="1"/>
       <c r="M5" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="N5" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="N5" s="1" t="s">
-        <v>127</v>
-      </c>
       <c r="O5" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="P5" s="1"/>
       <c r="Q5" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="R5" s="1"/>
       <c r="S5" s="1"/>
@@ -5503,49 +5505,49 @@
     </row>
     <row r="6" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
+        <v>146</v>
+      </c>
+      <c r="B6" s="10" t="s">
         <v>147</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="C6" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="E6" s="11" t="s">
         <v>148</v>
       </c>
-      <c r="C6" s="9" t="s">
-        <v>108</v>
-      </c>
-      <c r="D6" s="9" t="s">
-        <v>119</v>
-      </c>
-      <c r="E6" s="11" t="s">
+      <c r="F6" s="10" t="s">
+        <v>143</v>
+      </c>
+      <c r="G6" s="10" t="s">
         <v>149</v>
       </c>
-      <c r="F6" s="10" t="s">
-        <v>144</v>
-      </c>
-      <c r="G6" s="10" t="s">
-        <v>150</v>
-      </c>
       <c r="H6" s="10" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I6" s="7" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="J6" s="9"/>
       <c r="K6" s="9" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="L6" s="9"/>
       <c r="M6" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="N6" s="9" t="s">
         <v>126</v>
       </c>
-      <c r="N6" s="9" t="s">
-        <v>127</v>
-      </c>
       <c r="O6" s="9" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="P6" s="9"/>
       <c r="Q6" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="R6" s="9"/>
       <c r="S6" s="9"/>
@@ -5562,49 +5564,49 @@
     </row>
     <row r="7" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="B7" s="7" t="s">
         <v>151</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="C7" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="E7" s="8" t="s">
         <v>152</v>
       </c>
-      <c r="C7" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="E7" s="8" t="s">
+      <c r="F7" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="G7" s="7" t="s">
         <v>153</v>
       </c>
-      <c r="F7" s="7" t="s">
-        <v>133</v>
-      </c>
-      <c r="G7" s="7" t="s">
+      <c r="H7" s="7" t="s">
         <v>154</v>
       </c>
-      <c r="H7" s="7" t="s">
-        <v>155</v>
-      </c>
       <c r="I7" s="7" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="J7" s="1"/>
       <c r="K7" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="L7" s="1"/>
       <c r="M7" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="N7" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="N7" s="1" t="s">
+      <c r="O7" s="1" t="s">
         <v>127</v>
-      </c>
-      <c r="O7" s="1" t="s">
-        <v>128</v>
       </c>
       <c r="P7" s="1"/>
       <c r="Q7" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="R7" s="1"/>
       <c r="S7" s="1"/>
@@ -5621,49 +5623,49 @@
     </row>
     <row r="8" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="B8" s="7" t="s">
         <v>156</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="C8" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="E8" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="C8" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="E8" s="8" t="s">
+      <c r="F8" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="G8" s="7" t="s">
         <v>158</v>
       </c>
-      <c r="F8" s="7" t="s">
-        <v>133</v>
-      </c>
-      <c r="G8" s="7" t="s">
+      <c r="H8" s="7" t="s">
         <v>159</v>
       </c>
-      <c r="H8" s="7" t="s">
-        <v>160</v>
-      </c>
       <c r="I8" s="7" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="J8" s="1"/>
       <c r="K8" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="L8" s="1"/>
       <c r="M8" s="1" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="N8" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="O8" s="1" t="s">
         <v>127</v>
-      </c>
-      <c r="O8" s="1" t="s">
-        <v>128</v>
       </c>
       <c r="P8" s="1"/>
       <c r="Q8" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="R8" s="1"/>
       <c r="S8" s="1"/>
@@ -5680,49 +5682,49 @@
     </row>
     <row r="9" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="B9" s="10" t="s">
         <v>162</v>
-      </c>
-      <c r="B9" s="10" t="s">
-        <v>163</v>
       </c>
       <c r="C9" s="9" t="s">
         <v>17</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E9" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="F9" s="10" t="s">
         <v>164</v>
       </c>
-      <c r="F9" s="10" t="s">
+      <c r="G9" s="10" t="s">
         <v>165</v>
       </c>
-      <c r="G9" s="10" t="s">
+      <c r="H9" s="10" t="s">
         <v>166</v>
       </c>
-      <c r="H9" s="10" t="s">
-        <v>167</v>
-      </c>
       <c r="I9" s="7" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="J9" s="9"/>
       <c r="K9" s="9" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="L9" s="9"/>
       <c r="M9" s="9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="N9" s="9" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="O9" s="9" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="P9" s="9"/>
       <c r="Q9" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="R9" s="9"/>
       <c r="S9" s="9"/>
@@ -5739,47 +5741,47 @@
     </row>
     <row r="10" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="B10" s="12" t="s">
         <v>169</v>
-      </c>
-      <c r="B10" s="12" t="s">
-        <v>170</v>
       </c>
       <c r="C10" s="13" t="s">
         <v>17</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E10" s="12" t="s">
+        <v>170</v>
+      </c>
+      <c r="F10" s="12" t="s">
         <v>171</v>
       </c>
-      <c r="F10" s="12" t="s">
+      <c r="G10" s="12" t="s">
         <v>172</v>
       </c>
-      <c r="G10" s="12" t="s">
-        <v>173</v>
-      </c>
       <c r="H10" s="14" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="I10" s="12"/>
       <c r="J10" s="12"/>
       <c r="K10" s="12" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="L10" s="12"/>
       <c r="M10" s="14" t="s">
+        <v>173</v>
+      </c>
+      <c r="N10" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="O10" s="14" t="s">
         <v>174</v>
-      </c>
-      <c r="N10" s="12" t="s">
-        <v>127</v>
-      </c>
-      <c r="O10" s="14" t="s">
-        <v>175</v>
       </c>
       <c r="P10" s="12"/>
       <c r="Q10" s="1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="R10" s="12"/>
       <c r="S10" s="12"/>
@@ -5796,47 +5798,47 @@
     </row>
     <row r="11" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="12" t="s">
+        <v>176</v>
+      </c>
+      <c r="B11" s="12" t="s">
         <v>177</v>
       </c>
-      <c r="B11" s="12" t="s">
+      <c r="C11" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="D11" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="E11" s="12" t="s">
+        <v>170</v>
+      </c>
+      <c r="F11" s="12" t="s">
+        <v>171</v>
+      </c>
+      <c r="G11" s="12" t="s">
         <v>178</v>
       </c>
-      <c r="C11" s="13" t="s">
-        <v>108</v>
-      </c>
-      <c r="D11" s="12" t="s">
-        <v>119</v>
-      </c>
-      <c r="E11" s="12" t="s">
-        <v>171</v>
-      </c>
-      <c r="F11" s="12" t="s">
-        <v>172</v>
-      </c>
-      <c r="G11" s="12" t="s">
+      <c r="H11" s="14" t="s">
         <v>179</v>
-      </c>
-      <c r="H11" s="14" t="s">
-        <v>180</v>
       </c>
       <c r="I11" s="12"/>
       <c r="J11" s="12"/>
       <c r="K11" s="12" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="L11" s="12"/>
       <c r="M11" s="14" t="s">
+        <v>173</v>
+      </c>
+      <c r="N11" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="O11" s="14" t="s">
         <v>174</v>
-      </c>
-      <c r="N11" s="12" t="s">
-        <v>127</v>
-      </c>
-      <c r="O11" s="14" t="s">
-        <v>175</v>
       </c>
       <c r="P11" s="12"/>
       <c r="Q11" s="1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="R11" s="12"/>
       <c r="S11" s="12"/>
@@ -5853,47 +5855,47 @@
     </row>
     <row r="12" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="B12" s="12" t="s">
         <v>181</v>
       </c>
-      <c r="B12" s="12" t="s">
+      <c r="C12" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="D12" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="E12" s="12" t="s">
+        <v>170</v>
+      </c>
+      <c r="F12" s="12" t="s">
+        <v>171</v>
+      </c>
+      <c r="G12" s="12" t="s">
         <v>182</v>
       </c>
-      <c r="C12" s="13" t="s">
-        <v>108</v>
-      </c>
-      <c r="D12" s="12" t="s">
-        <v>119</v>
-      </c>
-      <c r="E12" s="12" t="s">
-        <v>171</v>
-      </c>
-      <c r="F12" s="12" t="s">
-        <v>172</v>
-      </c>
-      <c r="G12" s="12" t="s">
-        <v>183</v>
-      </c>
       <c r="H12" s="14" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="I12" s="12"/>
       <c r="J12" s="12"/>
       <c r="K12" s="12" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="L12" s="12"/>
       <c r="M12" s="14" t="s">
+        <v>173</v>
+      </c>
+      <c r="N12" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="O12" s="14" t="s">
         <v>174</v>
-      </c>
-      <c r="N12" s="12" t="s">
-        <v>127</v>
-      </c>
-      <c r="O12" s="14" t="s">
-        <v>175</v>
       </c>
       <c r="P12" s="12"/>
       <c r="Q12" s="1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="R12" s="12"/>
       <c r="S12" s="12"/>
@@ -5910,47 +5912,47 @@
     </row>
     <row r="13" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="12" t="s">
+        <v>183</v>
+      </c>
+      <c r="B13" s="12" t="s">
         <v>184</v>
-      </c>
-      <c r="B13" s="12" t="s">
-        <v>185</v>
       </c>
       <c r="C13" s="13" t="s">
         <v>17</v>
       </c>
       <c r="D13" s="12" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E13" s="12" t="s">
+        <v>170</v>
+      </c>
+      <c r="F13" s="12" t="s">
         <v>171</v>
       </c>
-      <c r="F13" s="12" t="s">
-        <v>172</v>
-      </c>
       <c r="G13" s="12" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="H13" s="14" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="I13" s="12"/>
       <c r="J13" s="12"/>
       <c r="K13" s="12" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="L13" s="12"/>
       <c r="M13" s="14" t="s">
+        <v>173</v>
+      </c>
+      <c r="N13" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="O13" s="14" t="s">
         <v>174</v>
-      </c>
-      <c r="N13" s="12" t="s">
-        <v>127</v>
-      </c>
-      <c r="O13" s="14" t="s">
-        <v>175</v>
       </c>
       <c r="P13" s="12"/>
       <c r="Q13" s="1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="R13" s="12"/>
       <c r="S13" s="12"/>
@@ -5967,47 +5969,47 @@
     </row>
     <row r="14" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="12" t="s">
+        <v>186</v>
+      </c>
+      <c r="B14" s="12" t="s">
         <v>187</v>
-      </c>
-      <c r="B14" s="12" t="s">
-        <v>188</v>
       </c>
       <c r="C14" s="13" t="s">
         <v>17</v>
       </c>
       <c r="D14" s="12" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E14" s="12" t="s">
+        <v>170</v>
+      </c>
+      <c r="F14" s="12" t="s">
         <v>171</v>
       </c>
-      <c r="F14" s="12" t="s">
-        <v>172</v>
-      </c>
       <c r="G14" s="12" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="H14" s="14" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="I14" s="12"/>
       <c r="J14" s="12"/>
       <c r="K14" s="12" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="L14" s="12"/>
       <c r="M14" s="14" t="s">
+        <v>173</v>
+      </c>
+      <c r="N14" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="O14" s="14" t="s">
         <v>174</v>
-      </c>
-      <c r="N14" s="12" t="s">
-        <v>127</v>
-      </c>
-      <c r="O14" s="14" t="s">
-        <v>175</v>
       </c>
       <c r="P14" s="12"/>
       <c r="Q14" s="1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="R14" s="12"/>
       <c r="S14" s="12"/>
@@ -6024,47 +6026,47 @@
     </row>
     <row r="15" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="12" t="s">
+        <v>189</v>
+      </c>
+      <c r="B15" s="12" t="s">
         <v>190</v>
-      </c>
-      <c r="B15" s="12" t="s">
-        <v>191</v>
       </c>
       <c r="C15" s="13" t="s">
         <v>17</v>
       </c>
       <c r="D15" s="12" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E15" s="12" t="s">
+        <v>170</v>
+      </c>
+      <c r="F15" s="12" t="s">
         <v>171</v>
       </c>
-      <c r="F15" s="12" t="s">
-        <v>172</v>
-      </c>
       <c r="G15" s="12" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="H15" s="14" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="I15" s="12"/>
       <c r="J15" s="12"/>
       <c r="K15" s="12" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="L15" s="12"/>
       <c r="M15" s="14" t="s">
+        <v>192</v>
+      </c>
+      <c r="N15" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="O15" s="14" t="s">
         <v>193</v>
-      </c>
-      <c r="N15" s="12" t="s">
-        <v>127</v>
-      </c>
-      <c r="O15" s="14" t="s">
-        <v>194</v>
       </c>
       <c r="P15" s="12"/>
       <c r="Q15" s="1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="R15" s="12"/>
       <c r="S15" s="12"/>
@@ -6081,47 +6083,47 @@
     </row>
     <row r="16" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="12" t="s">
+        <v>194</v>
+      </c>
+      <c r="B16" s="12" t="s">
         <v>195</v>
-      </c>
-      <c r="B16" s="12" t="s">
-        <v>196</v>
       </c>
       <c r="C16" s="13" t="s">
         <v>17</v>
       </c>
       <c r="D16" s="12" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E16" s="12" t="s">
+        <v>170</v>
+      </c>
+      <c r="F16" s="12" t="s">
         <v>171</v>
       </c>
-      <c r="F16" s="12" t="s">
-        <v>172</v>
-      </c>
       <c r="G16" s="12" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="H16" s="14" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="I16" s="12"/>
       <c r="J16" s="12"/>
       <c r="K16" s="12" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="L16" s="12"/>
       <c r="M16" s="14" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="N16" s="12" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="O16" s="14" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="P16" s="12"/>
       <c r="Q16" s="1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="R16" s="12"/>
       <c r="S16" s="12"/>
@@ -6138,192 +6140,192 @@
     </row>
     <row r="17" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="B17" s="3" t="s">
         <v>199</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>200</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>17</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F17" s="3" t="s">
+        <v>200</v>
+      </c>
+      <c r="G17" s="3" t="s">
         <v>201</v>
       </c>
-      <c r="G17" s="3" t="s">
+      <c r="H17" s="4" t="s">
         <v>202</v>
       </c>
-      <c r="H17" s="4" t="s">
+      <c r="J17" s="3" t="s">
         <v>203</v>
       </c>
-      <c r="J17" s="3" t="s">
-        <v>204</v>
-      </c>
       <c r="K17" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="L17" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M17" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="N17" s="3" t="s">
         <v>205</v>
       </c>
-      <c r="N17" s="3" t="s">
+      <c r="O17" s="4" t="s">
         <v>206</v>
       </c>
-      <c r="O17" s="4" t="s">
+      <c r="Q17" s="1" t="s">
         <v>207</v>
-      </c>
-      <c r="Q17" s="1" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="18" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
+        <v>208</v>
+      </c>
+      <c r="B18" s="3" t="s">
         <v>209</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>210</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>17</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E18" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="F18" s="3" t="s">
         <v>211</v>
       </c>
-      <c r="F18" s="3" t="s">
-        <v>212</v>
-      </c>
       <c r="G18" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="H18" s="4" t="s">
         <v>202</v>
       </c>
-      <c r="H18" s="4" t="s">
+      <c r="J18" s="3" t="s">
         <v>203</v>
       </c>
-      <c r="J18" s="3" t="s">
-        <v>204</v>
-      </c>
       <c r="K18" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="L18" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M18" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="N18" s="3" t="s">
         <v>205</v>
       </c>
-      <c r="N18" s="3" t="s">
+      <c r="O18" s="4" t="s">
         <v>206</v>
       </c>
-      <c r="O18" s="4" t="s">
+      <c r="Q18" s="1" t="s">
         <v>207</v>
-      </c>
-      <c r="Q18" s="1" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="19" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
+        <v>212</v>
+      </c>
+      <c r="B19" s="3" t="s">
         <v>213</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>214</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>17</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F19" s="3" t="s">
+        <v>214</v>
+      </c>
+      <c r="G19" s="3" t="s">
         <v>215</v>
       </c>
-      <c r="G19" s="3" t="s">
+      <c r="H19" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="J19" s="3" t="s">
         <v>216</v>
       </c>
-      <c r="H19" s="4" t="s">
-        <v>203</v>
-      </c>
-      <c r="J19" s="3" t="s">
-        <v>217</v>
-      </c>
       <c r="K19" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="L19" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M19" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="N19" s="3" t="s">
         <v>205</v>
       </c>
-      <c r="N19" s="3" t="s">
+      <c r="O19" s="4" t="s">
         <v>206</v>
       </c>
-      <c r="O19" s="4" t="s">
+      <c r="Q19" s="1" t="s">
         <v>207</v>
-      </c>
-      <c r="Q19" s="1" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="20" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="B20" s="15" t="s">
         <v>218</v>
       </c>
-      <c r="B20" s="15" t="s">
+      <c r="C20" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="D20" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="E20" s="15" t="s">
+        <v>210</v>
+      </c>
+      <c r="F20" s="15" t="s">
+        <v>200</v>
+      </c>
+      <c r="G20" s="15" t="s">
         <v>219</v>
       </c>
-      <c r="C20" s="9" t="s">
-        <v>108</v>
-      </c>
-      <c r="D20" s="15" t="s">
-        <v>119</v>
-      </c>
-      <c r="E20" s="15" t="s">
-        <v>211</v>
-      </c>
-      <c r="F20" s="15" t="s">
-        <v>201</v>
-      </c>
-      <c r="G20" s="15" t="s">
+      <c r="H20" s="15" t="s">
         <v>220</v>
-      </c>
-      <c r="H20" s="15" t="s">
-        <v>221</v>
       </c>
       <c r="I20" s="15"/>
       <c r="J20" s="15" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="K20" s="15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="L20" s="15" t="s">
         <v>23</v>
       </c>
       <c r="M20" s="16" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="N20" s="15" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="O20" s="4" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="P20" s="15"/>
       <c r="Q20" s="1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="R20" s="15"/>
       <c r="S20" s="15"/>
@@ -6340,51 +6342,51 @@
     </row>
     <row r="21" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="17" t="s">
+        <v>223</v>
+      </c>
+      <c r="B21" s="17" t="s">
         <v>224</v>
-      </c>
-      <c r="B21" s="17" t="s">
-        <v>225</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>17</v>
       </c>
       <c r="D21" s="18" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E21" s="18" t="s">
+        <v>225</v>
+      </c>
+      <c r="F21" s="17" t="s">
         <v>226</v>
       </c>
-      <c r="F21" s="17" t="s">
+      <c r="G21" s="19" t="s">
         <v>227</v>
       </c>
-      <c r="G21" s="19" t="s">
+      <c r="H21" s="17" t="s">
         <v>228</v>
       </c>
-      <c r="H21" s="17" t="s">
+      <c r="I21" s="20" t="s">
         <v>229</v>
-      </c>
-      <c r="I21" s="20" t="s">
-        <v>230</v>
       </c>
       <c r="J21" s="2"/>
       <c r="K21" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="L21" s="2"/>
       <c r="M21" s="21" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="N21" s="17" t="s">
         <v>44</v>
       </c>
       <c r="O21" s="18" t="s">
+        <v>231</v>
+      </c>
+      <c r="P21" s="22" t="s">
         <v>232</v>
       </c>
-      <c r="P21" s="22" t="s">
-        <v>233</v>
-      </c>
       <c r="Q21" s="1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="R21" s="2"/>
       <c r="S21" s="2"/>
@@ -6401,237 +6403,237 @@
     </row>
     <row r="22" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="B22" s="3" t="s">
         <v>234</v>
       </c>
-      <c r="B22" s="3" t="s">
+      <c r="C22" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="E22" s="20" t="s">
         <v>235</v>
       </c>
-      <c r="C22" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="D22" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="E22" s="20" t="s">
+      <c r="F22" s="20" t="s">
         <v>236</v>
       </c>
-      <c r="F22" s="20" t="s">
+      <c r="G22" s="20" t="s">
         <v>237</v>
       </c>
-      <c r="G22" s="20" t="s">
+      <c r="H22" s="23" t="s">
         <v>238</v>
       </c>
-      <c r="H22" s="23" t="s">
+      <c r="I22" s="20" t="s">
+        <v>229</v>
+      </c>
+      <c r="K22" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="M22" s="4" t="s">
         <v>239</v>
       </c>
-      <c r="I22" s="20" t="s">
-        <v>230</v>
-      </c>
-      <c r="K22" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="M22" s="4" t="s">
+      <c r="N22" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="O22" s="4" t="s">
         <v>240</v>
       </c>
-      <c r="N22" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="O22" s="4" t="s">
-        <v>241</v>
-      </c>
       <c r="P22" s="22" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="Q22" s="1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="23" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="B23" s="3" t="s">
         <v>242</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="C23" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="E23" s="20" t="s">
+        <v>235</v>
+      </c>
+      <c r="F23" s="24" t="s">
         <v>243</v>
       </c>
-      <c r="C23" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="D23" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="E23" s="20" t="s">
-        <v>236</v>
-      </c>
-      <c r="F23" s="24" t="s">
+      <c r="G23" s="20" t="s">
         <v>244</v>
       </c>
-      <c r="G23" s="20" t="s">
-        <v>245</v>
-      </c>
       <c r="H23" s="23" t="s">
+        <v>238</v>
+      </c>
+      <c r="I23" s="20" t="s">
+        <v>229</v>
+      </c>
+      <c r="K23" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="M23" s="4" t="s">
         <v>239</v>
       </c>
-      <c r="I23" s="20" t="s">
-        <v>230</v>
-      </c>
-      <c r="K23" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="M23" s="4" t="s">
+      <c r="N23" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="O23" s="4" t="s">
         <v>240</v>
       </c>
-      <c r="N23" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="O23" s="4" t="s">
-        <v>241</v>
-      </c>
       <c r="P23" s="22" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="Q23" s="1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="24" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="B24" s="3" t="s">
         <v>246</v>
       </c>
-      <c r="B24" s="3" t="s">
+      <c r="C24" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="E24" s="20" t="s">
         <v>247</v>
       </c>
-      <c r="C24" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="D24" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="E24" s="20" t="s">
+      <c r="F24" s="20" t="s">
         <v>248</v>
       </c>
-      <c r="F24" s="20" t="s">
+      <c r="G24" s="3" t="s">
         <v>249</v>
       </c>
-      <c r="G24" s="3" t="s">
+      <c r="H24" s="23" t="s">
         <v>250</v>
       </c>
-      <c r="H24" s="23" t="s">
+      <c r="I24" s="20" t="s">
+        <v>229</v>
+      </c>
+      <c r="K24" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="M24" s="4" t="s">
         <v>251</v>
       </c>
-      <c r="I24" s="20" t="s">
-        <v>230</v>
-      </c>
-      <c r="K24" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="M24" s="4" t="s">
-        <v>252</v>
-      </c>
       <c r="N24" s="3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="O24" s="4"/>
       <c r="P24" s="22" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="Q24" s="1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="25" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="B25" s="3" t="s">
         <v>253</v>
       </c>
-      <c r="B25" s="3" t="s">
+      <c r="C25" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="E25" s="20" t="s">
+        <v>235</v>
+      </c>
+      <c r="F25" s="20" t="s">
         <v>254</v>
       </c>
-      <c r="C25" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="D25" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="E25" s="20" t="s">
-        <v>236</v>
-      </c>
-      <c r="F25" s="20" t="s">
+      <c r="G25" s="3" t="s">
         <v>255</v>
       </c>
-      <c r="G25" s="3" t="s">
+      <c r="H25" s="1" t="s">
         <v>256</v>
       </c>
-      <c r="H25" s="1" t="s">
+      <c r="I25" s="20" t="s">
+        <v>229</v>
+      </c>
+      <c r="K25" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="M25" s="4" t="s">
         <v>257</v>
       </c>
-      <c r="I25" s="20" t="s">
-        <v>230</v>
-      </c>
-      <c r="K25" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="M25" s="4" t="s">
-        <v>258</v>
-      </c>
       <c r="N25" s="3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="O25" s="4" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="P25" s="22" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="Q25" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="26" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="15" t="s">
+        <v>258</v>
+      </c>
+      <c r="B26" s="15" t="s">
         <v>259</v>
       </c>
-      <c r="B26" s="15" t="s">
+      <c r="C26" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="D26" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="E26" s="25" t="s">
+        <v>235</v>
+      </c>
+      <c r="F26" s="25" t="s">
         <v>260</v>
       </c>
-      <c r="C26" s="9" t="s">
-        <v>108</v>
-      </c>
-      <c r="D26" s="15" t="s">
-        <v>119</v>
-      </c>
-      <c r="E26" s="25" t="s">
-        <v>236</v>
-      </c>
-      <c r="F26" s="25" t="s">
+      <c r="G26" s="15" t="s">
         <v>261</v>
       </c>
-      <c r="G26" s="15" t="s">
-        <v>262</v>
-      </c>
       <c r="H26" s="9" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="I26" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="J26" s="15"/>
       <c r="K26" s="15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="L26" s="15"/>
       <c r="M26" s="16" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="N26" s="15" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="O26" s="16" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="P26" s="22" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="Q26" s="1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="R26" s="15"/>
       <c r="S26" s="15"/>
@@ -6648,336 +6650,336 @@
     </row>
     <row r="27" spans="1:29" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
+        <v>262</v>
+      </c>
+      <c r="B27" s="3" t="s">
         <v>263</v>
       </c>
-      <c r="B27" s="3" t="s">
+      <c r="C27" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="D27" s="3" t="s">
         <v>264</v>
       </c>
-      <c r="C27" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="D27" s="3" t="s">
+      <c r="E27" s="3" t="s">
         <v>265</v>
       </c>
-      <c r="E27" s="3" t="s">
+      <c r="F27" s="3" t="s">
         <v>266</v>
       </c>
-      <c r="F27" s="3" t="s">
+      <c r="G27" s="3" t="s">
         <v>267</v>
       </c>
-      <c r="G27" s="3" t="s">
+      <c r="H27" s="4" t="s">
         <v>268</v>
       </c>
-      <c r="H27" s="4" t="s">
+      <c r="K27" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="M27" s="4" t="s">
         <v>269</v>
       </c>
-      <c r="K27" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="M27" s="4" t="s">
+      <c r="N27" s="3" t="s">
         <v>270</v>
       </c>
-      <c r="N27" s="3" t="s">
+      <c r="O27" s="4" t="s">
         <v>271</v>
       </c>
-      <c r="O27" s="4" t="s">
-        <v>272</v>
-      </c>
       <c r="Q27" s="1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="28" spans="1:29" ht="66.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
+        <v>272</v>
+      </c>
+      <c r="B28" s="3" t="s">
         <v>273</v>
       </c>
-      <c r="B28" s="3" t="s">
+      <c r="C28" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>264</v>
+      </c>
+      <c r="E28" s="3" t="s">
         <v>274</v>
       </c>
-      <c r="C28" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="D28" s="3" t="s">
-        <v>265</v>
-      </c>
-      <c r="E28" s="3" t="s">
+      <c r="F28" s="3" t="s">
         <v>275</v>
       </c>
-      <c r="F28" s="3" t="s">
+      <c r="G28" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="G28" s="3" t="s">
+      <c r="H28" s="4" t="s">
         <v>277</v>
       </c>
-      <c r="H28" s="4" t="s">
+      <c r="K28" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="M28" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="N28" s="3" t="s">
+        <v>270</v>
+      </c>
+      <c r="O28" s="4" t="s">
         <v>278</v>
       </c>
-      <c r="K28" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="M28" s="4" t="s">
-        <v>270</v>
-      </c>
-      <c r="N28" s="3" t="s">
-        <v>271</v>
-      </c>
-      <c r="O28" s="4" t="s">
-        <v>279</v>
-      </c>
       <c r="Q28" s="1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="29" spans="1:29" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="B29" s="3" t="s">
         <v>280</v>
-      </c>
-      <c r="B29" s="3" t="s">
-        <v>281</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>17</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="E29" s="3" t="s">
+        <v>281</v>
+      </c>
+      <c r="F29" s="3" t="s">
         <v>282</v>
-      </c>
-      <c r="F29" s="3" t="s">
-        <v>283</v>
       </c>
       <c r="G29" s="3" t="s">
         <v>23</v>
       </c>
       <c r="H29" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="K29" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="M29" s="4" t="s">
         <v>284</v>
       </c>
-      <c r="K29" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="M29" s="4" t="s">
-        <v>285</v>
-      </c>
       <c r="N29" s="3" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="O29" s="4" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="Q29" s="1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="30" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
+        <v>285</v>
+      </c>
+      <c r="B30" s="3" t="s">
         <v>286</v>
-      </c>
-      <c r="B30" s="3" t="s">
-        <v>287</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>17</v>
       </c>
       <c r="D30" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="E30" s="3" t="s">
         <v>288</v>
       </c>
-      <c r="E30" s="3" t="s">
+      <c r="F30" s="3" t="s">
         <v>289</v>
       </c>
-      <c r="F30" s="3" t="s">
+      <c r="G30" s="3" t="s">
         <v>290</v>
       </c>
-      <c r="G30" s="3" t="s">
+      <c r="H30" s="23" t="s">
         <v>291</v>
       </c>
-      <c r="H30" s="23" t="s">
+      <c r="K30" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="M30" s="4" t="s">
         <v>292</v>
       </c>
-      <c r="K30" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="M30" s="4" t="s">
+      <c r="O30" s="4" t="s">
         <v>293</v>
       </c>
-      <c r="O30" s="4" t="s">
-        <v>294</v>
-      </c>
       <c r="Q30" s="1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="31" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
+        <v>294</v>
+      </c>
+      <c r="B31" s="3" t="s">
         <v>295</v>
-      </c>
-      <c r="B31" s="3" t="s">
-        <v>296</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>17</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="E31" s="3" t="s">
         <v>23</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="G31" s="3" t="s">
         <v>23</v>
       </c>
       <c r="H31" s="23" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="K31" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="M31" s="4" t="s">
+        <v>292</v>
+      </c>
+      <c r="O31" s="4" t="s">
         <v>293</v>
       </c>
-      <c r="O31" s="4" t="s">
-        <v>294</v>
-      </c>
       <c r="Q31" s="1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="32" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
+        <v>298</v>
+      </c>
+      <c r="B32" s="3" t="s">
         <v>299</v>
-      </c>
-      <c r="B32" s="3" t="s">
-        <v>300</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>17</v>
       </c>
       <c r="D32" s="3" t="s">
+        <v>300</v>
+      </c>
+      <c r="E32" s="3" t="s">
         <v>301</v>
       </c>
-      <c r="E32" s="3" t="s">
+      <c r="F32" s="3" t="s">
         <v>302</v>
       </c>
-      <c r="F32" s="3" t="s">
+      <c r="G32" s="3" t="s">
         <v>303</v>
       </c>
-      <c r="G32" s="3" t="s">
+      <c r="H32" s="23" t="s">
         <v>304</v>
       </c>
-      <c r="H32" s="23" t="s">
-        <v>305</v>
-      </c>
       <c r="I32" s="26" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="J32" s="3" t="s">
         <v>23</v>
       </c>
       <c r="K32" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="M32" s="4" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="O32" s="4" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="Q32" s="1" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="33" spans="1:29" ht="55.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
+        <v>306</v>
+      </c>
+      <c r="B33" s="3" t="s">
         <v>307</v>
-      </c>
-      <c r="B33" s="3" t="s">
-        <v>308</v>
       </c>
       <c r="C33" s="1" t="s">
         <v>17</v>
       </c>
       <c r="D33" s="3" t="s">
+        <v>308</v>
+      </c>
+      <c r="E33" s="3" t="s">
         <v>309</v>
       </c>
-      <c r="E33" s="3" t="s">
+      <c r="F33" s="3" t="s">
         <v>310</v>
       </c>
-      <c r="F33" s="3" t="s">
+      <c r="G33" s="27" t="s">
         <v>311</v>
       </c>
-      <c r="G33" s="27" t="s">
+      <c r="H33" s="23" t="s">
         <v>312</v>
       </c>
-      <c r="H33" s="23" t="s">
+      <c r="J33" s="3" t="s">
         <v>313</v>
       </c>
-      <c r="J33" s="3" t="s">
+      <c r="K33" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="M33" s="4" t="s">
         <v>314</v>
       </c>
-      <c r="K33" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="M33" s="4" t="s">
+      <c r="N33" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="O33" s="4" t="s">
         <v>315</v>
       </c>
-      <c r="N33" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="O33" s="4" t="s">
-        <v>316</v>
-      </c>
       <c r="Q33" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="34" spans="1:29" ht="63.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="28" t="s">
+        <v>316</v>
+      </c>
+      <c r="B34" s="3" t="s">
         <v>317</v>
       </c>
-      <c r="B34" s="3" t="s">
+      <c r="C34" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="E34" s="28" t="s">
         <v>318</v>
       </c>
-      <c r="C34" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="D34" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="E34" s="28" t="s">
+      <c r="F34" s="28" t="s">
         <v>319</v>
       </c>
-      <c r="F34" s="28" t="s">
+      <c r="G34" s="28" t="s">
         <v>320</v>
       </c>
-      <c r="G34" s="28" t="s">
+      <c r="H34" s="29" t="s">
         <v>321</v>
-      </c>
-      <c r="H34" s="29" t="s">
-        <v>322</v>
       </c>
       <c r="I34" s="28"/>
       <c r="J34" s="28" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="K34" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="L34" s="28"/>
       <c r="M34" s="30" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="N34" s="28" t="s">
         <v>44</v>
       </c>
       <c r="O34" s="29" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="P34" s="28"/>
       <c r="Q34" s="1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="R34" s="28"/>
       <c r="S34" s="28"/>
@@ -6994,49 +6996,49 @@
     </row>
     <row r="35" spans="1:29" ht="67.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="28" t="s">
+        <v>323</v>
+      </c>
+      <c r="B35" s="3" t="s">
         <v>324</v>
       </c>
-      <c r="B35" s="3" t="s">
+      <c r="C35" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="E35" s="28" t="s">
+        <v>318</v>
+      </c>
+      <c r="F35" s="28" t="s">
+        <v>319</v>
+      </c>
+      <c r="G35" s="28" t="s">
         <v>325</v>
       </c>
-      <c r="C35" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="D35" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="E35" s="28" t="s">
-        <v>319</v>
-      </c>
-      <c r="F35" s="28" t="s">
-        <v>320</v>
-      </c>
-      <c r="G35" s="28" t="s">
-        <v>326</v>
-      </c>
       <c r="H35" s="29" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="I35" s="28"/>
       <c r="J35" s="28" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="K35" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="L35" s="28"/>
       <c r="M35" s="30" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="N35" s="28" t="s">
         <v>44</v>
       </c>
       <c r="O35" s="29" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="P35" s="28"/>
       <c r="Q35" s="1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="R35" s="28"/>
       <c r="S35" s="28"/>
@@ -7053,93 +7055,93 @@
     </row>
     <row r="36" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
+        <v>326</v>
+      </c>
+      <c r="B36" s="3" t="s">
         <v>327</v>
-      </c>
-      <c r="B36" s="3" t="s">
-        <v>328</v>
       </c>
       <c r="C36" s="1" t="s">
         <v>17</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E36" s="31" t="s">
+        <v>328</v>
+      </c>
+      <c r="F36" s="3" t="s">
         <v>329</v>
       </c>
-      <c r="F36" s="3" t="s">
+      <c r="G36" s="3" t="s">
         <v>330</v>
       </c>
-      <c r="G36" s="3" t="s">
+      <c r="H36" s="4" t="s">
         <v>331</v>
       </c>
-      <c r="H36" s="4" t="s">
+      <c r="J36" s="3" t="s">
+        <v>313</v>
+      </c>
+      <c r="K36" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="M36" s="27" t="s">
         <v>332</v>
-      </c>
-      <c r="J36" s="3" t="s">
-        <v>314</v>
-      </c>
-      <c r="K36" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="M36" s="27" t="s">
-        <v>333</v>
       </c>
       <c r="N36" s="3" t="s">
         <v>44</v>
       </c>
       <c r="O36" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="Q36" s="1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="37" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="28" t="s">
+        <v>333</v>
+      </c>
+      <c r="B37" s="28" t="s">
         <v>334</v>
-      </c>
-      <c r="B37" s="28" t="s">
-        <v>335</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>17</v>
       </c>
       <c r="D37" s="28" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E37" s="26" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="F37" s="28" t="s">
+        <v>335</v>
+      </c>
+      <c r="G37" s="28" t="s">
         <v>336</v>
       </c>
-      <c r="G37" s="28" t="s">
+      <c r="H37" s="32" t="s">
         <v>337</v>
-      </c>
-      <c r="H37" s="32" t="s">
-        <v>338</v>
       </c>
       <c r="I37" s="28"/>
       <c r="J37" s="28" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="K37" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="L37" s="28"/>
       <c r="M37" s="30" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="N37" s="28" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="O37" s="29" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="P37" s="28"/>
       <c r="Q37" s="1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="R37" s="28"/>
       <c r="S37" s="28"/>
@@ -7156,49 +7158,49 @@
     </row>
     <row r="38" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="28" t="s">
+        <v>339</v>
+      </c>
+      <c r="B38" s="28" t="s">
         <v>340</v>
       </c>
-      <c r="B38" s="28" t="s">
+      <c r="C38" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="D38" s="28" t="s">
+        <v>118</v>
+      </c>
+      <c r="E38" s="26" t="s">
+        <v>309</v>
+      </c>
+      <c r="F38" s="28" t="s">
         <v>341</v>
       </c>
-      <c r="C38" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="D38" s="28" t="s">
-        <v>119</v>
-      </c>
-      <c r="E38" s="26" t="s">
-        <v>310</v>
-      </c>
-      <c r="F38" s="28" t="s">
+      <c r="G38" s="28" t="s">
         <v>342</v>
       </c>
-      <c r="G38" s="28" t="s">
-        <v>343</v>
-      </c>
       <c r="H38" s="32" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="I38" s="28"/>
       <c r="J38" s="28" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="K38" s="28" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="L38" s="28"/>
       <c r="M38" s="30" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="N38" s="28" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="O38" s="29" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="P38" s="28"/>
       <c r="Q38" s="1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="R38" s="28"/>
       <c r="S38" s="28"/>

</xml_diff>

<commit_message>
test/update cart execution test cases.
</commit_message>
<xml_diff>
--- a/TestCases_Docs/ShoppingCart_TestCases.xlsx
+++ b/TestCases_Docs/ShoppingCart_TestCases.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lenovo\OneDrive\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\iti\QA\New folder\Clothing-Web-Portal\TestCases_Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{021F7BE5-8290-4F7E-A076-FB55A20AB955}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{193CCE82-1585-473C-963D-336FA7872E40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="11520" windowHeight="12360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cart Test Cases" sheetId="5" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1132" uniqueCount="367">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1132" uniqueCount="366">
   <si>
     <t>TesTCASE ID</t>
   </si>
@@ -1573,9 +1573,6 @@
   </si>
   <si>
     <t>Passed</t>
-  </si>
-  <si>
-    <t>Failed</t>
   </si>
   <si>
     <t>1- Email: gohary@mail.com
@@ -2111,328 +2108,6 @@
       </border>
     </dxf>
     <dxf>
-      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-        <family val="2"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color rgb="FF000000"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF000000"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF000000"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF000000"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <border>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
@@ -2751,6 +2426,328 @@
         </right>
         <top/>
         <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+        <family val="2"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
       </border>
     </dxf>
     <dxf>
@@ -2940,50 +2937,50 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{CA9B46E1-5155-4AAF-844B-BCD9CCA2EDF6}" name="Table17" displayName="Table17" ref="A1:O20" totalsRowShown="0" headerRowDxfId="21" dataDxfId="19" headerRowBorderDxfId="20" tableBorderDxfId="18" totalsRowBorderDxfId="17">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{CA9B46E1-5155-4AAF-844B-BCD9CCA2EDF6}" name="Table17" displayName="Table17" ref="A1:O20" totalsRowShown="0" headerRowDxfId="43" dataDxfId="41" headerRowBorderDxfId="42" tableBorderDxfId="40" totalsRowBorderDxfId="39">
   <autoFilter ref="A1:O20" xr:uid="{CA9B46E1-5155-4AAF-844B-BCD9CCA2EDF6}"/>
   <tableColumns count="15">
-    <tableColumn id="1" xr3:uid="{11F6C013-4C48-4E7A-B8F8-375AECFF097E}" name="TesTCASE ID" dataDxfId="16"/>
-    <tableColumn id="2" xr3:uid="{1B888F99-A907-40FC-B776-834DD24F6F57}" name="Test Cases Title " dataDxfId="15"/>
-    <tableColumn id="3" xr3:uid="{7853AC75-B7A3-4B9B-B597-0CC90E8D52BF}" name="valid/invalid" dataDxfId="14"/>
-    <tableColumn id="4" xr3:uid="{AAABAF80-25C1-4ACB-ADF4-7337AEA0E0A4}" name="Environment" dataDxfId="13"/>
-    <tableColumn id="5" xr3:uid="{050A3DD3-5C3B-40E3-B68A-DE6E46C20CD3}" name="Pre-condition" dataDxfId="12"/>
-    <tableColumn id="6" xr3:uid="{695FB61F-899E-47FB-AC04-D25E8F4EFFA9}" name="Steps" dataDxfId="11"/>
-    <tableColumn id="7" xr3:uid="{6AADAA49-15BA-4E3C-B63A-DDA3E7EF4C96}" name="Test Data" dataDxfId="10"/>
-    <tableColumn id="8" xr3:uid="{C1CE8F53-60B8-411D-A252-48EAF0B6899D}" name="Expected Results" dataDxfId="9"/>
-    <tableColumn id="9" xr3:uid="{5CBA8F0E-EFB2-441E-ABB2-C8AFC9733678}" name="Post Condition" dataDxfId="8"/>
-    <tableColumn id="10" xr3:uid="{F1F2F7F1-026F-45A0-971C-F5B647193AEB}" name="TC Status" dataDxfId="7"/>
-    <tableColumn id="11" xr3:uid="{C1B2E8E9-0DE1-4E62-B972-DE5006C951AE}" name="Attachment" dataDxfId="6"/>
-    <tableColumn id="12" xr3:uid="{3F1A62C0-FBFC-41F2-B1C9-42BCC073A738}" name="Requirement ID" dataDxfId="5"/>
-    <tableColumn id="13" xr3:uid="{FF0D4754-9DCA-4527-96A7-45E4EA4C6EED}" name="Type" dataDxfId="4"/>
-    <tableColumn id="14" xr3:uid="{CEE95E6B-C591-4C14-8305-FA320F301C59}" name="Tester" dataDxfId="3"/>
-    <tableColumn id="15" xr3:uid="{678D806D-10AD-4D08-AE9F-776FEBFD7C5C}" name="Comment" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{11F6C013-4C48-4E7A-B8F8-375AECFF097E}" name="TesTCASE ID" dataDxfId="38"/>
+    <tableColumn id="2" xr3:uid="{1B888F99-A907-40FC-B776-834DD24F6F57}" name="Test Cases Title " dataDxfId="37"/>
+    <tableColumn id="3" xr3:uid="{7853AC75-B7A3-4B9B-B597-0CC90E8D52BF}" name="valid/invalid" dataDxfId="36"/>
+    <tableColumn id="4" xr3:uid="{AAABAF80-25C1-4ACB-ADF4-7337AEA0E0A4}" name="Environment" dataDxfId="35"/>
+    <tableColumn id="5" xr3:uid="{050A3DD3-5C3B-40E3-B68A-DE6E46C20CD3}" name="Pre-condition" dataDxfId="34"/>
+    <tableColumn id="6" xr3:uid="{695FB61F-899E-47FB-AC04-D25E8F4EFFA9}" name="Steps" dataDxfId="33"/>
+    <tableColumn id="7" xr3:uid="{6AADAA49-15BA-4E3C-B63A-DDA3E7EF4C96}" name="Test Data" dataDxfId="32"/>
+    <tableColumn id="8" xr3:uid="{C1CE8F53-60B8-411D-A252-48EAF0B6899D}" name="Expected Results" dataDxfId="31"/>
+    <tableColumn id="9" xr3:uid="{5CBA8F0E-EFB2-441E-ABB2-C8AFC9733678}" name="Post Condition" dataDxfId="30"/>
+    <tableColumn id="10" xr3:uid="{F1F2F7F1-026F-45A0-971C-F5B647193AEB}" name="TC Status" dataDxfId="29"/>
+    <tableColumn id="11" xr3:uid="{C1B2E8E9-0DE1-4E62-B972-DE5006C951AE}" name="Attachment" dataDxfId="28"/>
+    <tableColumn id="12" xr3:uid="{3F1A62C0-FBFC-41F2-B1C9-42BCC073A738}" name="Requirement ID" dataDxfId="27"/>
+    <tableColumn id="13" xr3:uid="{FF0D4754-9DCA-4527-96A7-45E4EA4C6EED}" name="Type" dataDxfId="26"/>
+    <tableColumn id="14" xr3:uid="{CEE95E6B-C591-4C14-8305-FA320F301C59}" name="Tester" dataDxfId="25"/>
+    <tableColumn id="15" xr3:uid="{678D806D-10AD-4D08-AE9F-776FEBFD7C5C}" name="Comment" dataDxfId="24"/>
   </tableColumns>
   <tableStyleInfo name="Cart Test Cases-style" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="18" xr:uid="{7DE26239-599D-4E8A-B29E-9F20DE12A166}" name="Table1719" displayName="Table1719" ref="A1:Q20" totalsRowShown="0" headerRowDxfId="43" dataDxfId="41" headerRowBorderDxfId="42" tableBorderDxfId="40" totalsRowBorderDxfId="39">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="18" xr:uid="{7DE26239-599D-4E8A-B29E-9F20DE12A166}" name="Table1719" displayName="Table1719" ref="A1:Q20" totalsRowShown="0" headerRowDxfId="23" dataDxfId="21" headerRowBorderDxfId="22" tableBorderDxfId="20" totalsRowBorderDxfId="19">
   <autoFilter ref="A1:Q20" xr:uid="{CA9B46E1-5155-4AAF-844B-BCD9CCA2EDF6}"/>
   <tableColumns count="17">
-    <tableColumn id="1" xr3:uid="{6349AC1B-18C1-4513-A98D-74004451BE07}" name="TesTCASE ID" dataDxfId="38"/>
-    <tableColumn id="2" xr3:uid="{316A01E1-D06A-4667-AE3C-453DBC4B1054}" name="Test Cases Title " dataDxfId="37"/>
-    <tableColumn id="3" xr3:uid="{8F7A3C5E-7DAA-4BE5-BB4C-4242660A0347}" name="valid/invalid" dataDxfId="36"/>
-    <tableColumn id="4" xr3:uid="{6F77ADFD-1C3F-4A08-A6E4-478BE3CD7F59}" name="Environment" dataDxfId="35"/>
-    <tableColumn id="5" xr3:uid="{519F839C-1B74-4449-9BE1-EDCA27C25137}" name="Pre-condition" dataDxfId="34"/>
-    <tableColumn id="6" xr3:uid="{F29F0414-7871-4D01-A1DD-A280EE6716F5}" name="Steps" dataDxfId="33"/>
-    <tableColumn id="7" xr3:uid="{2749E69B-C03F-4456-97F1-16E4C7DAB4C8}" name="Test Data" dataDxfId="32"/>
-    <tableColumn id="8" xr3:uid="{10DFC294-FAB0-4D43-8B83-7C0CE4E11BE0}" name="Expected Results" dataDxfId="31"/>
-    <tableColumn id="16" xr3:uid="{2D24DDBD-5A02-4264-B89B-27175D91D43D}" name="Actual result" dataDxfId="30"/>
-    <tableColumn id="9" xr3:uid="{B771E747-8E01-4980-9B14-221C5B00CF89}" name="Post Condition" dataDxfId="29"/>
-    <tableColumn id="10" xr3:uid="{903AF337-308B-4432-90B3-453B150C8696}" name="TC Status" dataDxfId="28"/>
-    <tableColumn id="11" xr3:uid="{DA7982CC-CFB4-46EF-8D7D-498270ACE130}" name="Attachment" dataDxfId="27"/>
-    <tableColumn id="12" xr3:uid="{C3C4BBD3-BE51-4BB4-A9C8-4688454A9D7B}" name="Requirement ID" dataDxfId="26"/>
-    <tableColumn id="13" xr3:uid="{6FFDB195-604A-4141-B2B3-FB2EBCCF9EE1}" name="Type" dataDxfId="25"/>
-    <tableColumn id="14" xr3:uid="{0C076CE8-316D-4323-B69F-E0CA15A82960}" name="Tester" dataDxfId="24"/>
-    <tableColumn id="17" xr3:uid="{C124139E-C07E-4913-834E-C22FF51CDDC5}" name="Execution_Status" dataDxfId="23"/>
-    <tableColumn id="15" xr3:uid="{7B9BAC1F-276D-47AE-B4F7-FBBDF0CA5C1C}" name="Comment" dataDxfId="22"/>
+    <tableColumn id="1" xr3:uid="{6349AC1B-18C1-4513-A98D-74004451BE07}" name="TesTCASE ID" dataDxfId="18"/>
+    <tableColumn id="2" xr3:uid="{316A01E1-D06A-4667-AE3C-453DBC4B1054}" name="Test Cases Title " dataDxfId="17"/>
+    <tableColumn id="3" xr3:uid="{8F7A3C5E-7DAA-4BE5-BB4C-4242660A0347}" name="valid/invalid" dataDxfId="16"/>
+    <tableColumn id="4" xr3:uid="{6F77ADFD-1C3F-4A08-A6E4-478BE3CD7F59}" name="Environment" dataDxfId="15"/>
+    <tableColumn id="5" xr3:uid="{519F839C-1B74-4449-9BE1-EDCA27C25137}" name="Pre-condition" dataDxfId="14"/>
+    <tableColumn id="6" xr3:uid="{F29F0414-7871-4D01-A1DD-A280EE6716F5}" name="Steps" dataDxfId="13"/>
+    <tableColumn id="7" xr3:uid="{2749E69B-C03F-4456-97F1-16E4C7DAB4C8}" name="Test Data" dataDxfId="12"/>
+    <tableColumn id="8" xr3:uid="{10DFC294-FAB0-4D43-8B83-7C0CE4E11BE0}" name="Expected Results" dataDxfId="11"/>
+    <tableColumn id="16" xr3:uid="{2D24DDBD-5A02-4264-B89B-27175D91D43D}" name="Actual result" dataDxfId="10"/>
+    <tableColumn id="9" xr3:uid="{B771E747-8E01-4980-9B14-221C5B00CF89}" name="Post Condition" dataDxfId="9"/>
+    <tableColumn id="10" xr3:uid="{903AF337-308B-4432-90B3-453B150C8696}" name="TC Status" dataDxfId="8"/>
+    <tableColumn id="11" xr3:uid="{DA7982CC-CFB4-46EF-8D7D-498270ACE130}" name="Attachment" dataDxfId="7"/>
+    <tableColumn id="12" xr3:uid="{C3C4BBD3-BE51-4BB4-A9C8-4688454A9D7B}" name="Requirement ID" dataDxfId="6"/>
+    <tableColumn id="13" xr3:uid="{6FFDB195-604A-4141-B2B3-FB2EBCCF9EE1}" name="Type" dataDxfId="5"/>
+    <tableColumn id="14" xr3:uid="{0C076CE8-316D-4323-B69F-E0CA15A82960}" name="Tester" dataDxfId="4"/>
+    <tableColumn id="17" xr3:uid="{C124139E-C07E-4913-834E-C22FF51CDDC5}" name="Execution_Status" dataDxfId="3"/>
+    <tableColumn id="15" xr3:uid="{7B9BAC1F-276D-47AE-B4F7-FBBDF0CA5C1C}" name="Comment" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="Cart Test Cases-style" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3274,7 +3271,7 @@
         <v>20</v>
       </c>
       <c r="G2" s="53" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="H2" s="42" t="s">
         <v>21</v>
@@ -3319,7 +3316,7 @@
         <v>29</v>
       </c>
       <c r="G3" s="53" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="H3" s="42" t="s">
         <v>30</v>
@@ -3364,7 +3361,7 @@
         <v>33</v>
       </c>
       <c r="G4" s="53" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="H4" s="42" t="s">
         <v>34</v>
@@ -3409,7 +3406,7 @@
         <v>38</v>
       </c>
       <c r="G5" s="53" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="H5" s="42" t="s">
         <v>39</v>
@@ -3454,7 +3451,7 @@
         <v>42</v>
       </c>
       <c r="G6" s="53" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="H6" s="42" t="s">
         <v>43</v>
@@ -3499,7 +3496,7 @@
         <v>47</v>
       </c>
       <c r="G7" s="53" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="H7" s="42" t="s">
         <v>48</v>
@@ -3544,7 +3541,7 @@
         <v>51</v>
       </c>
       <c r="G8" s="53" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="H8" s="42" t="s">
         <v>52</v>
@@ -3589,7 +3586,7 @@
         <v>55</v>
       </c>
       <c r="G9" s="53" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="H9" s="42" t="s">
         <v>56</v>
@@ -3634,7 +3631,7 @@
         <v>61</v>
       </c>
       <c r="G10" s="53" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="H10" s="42" t="s">
         <v>62</v>
@@ -3679,7 +3676,7 @@
         <v>66</v>
       </c>
       <c r="G11" s="53" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="H11" s="42" t="s">
         <v>67</v>
@@ -3718,13 +3715,13 @@
         <v>18</v>
       </c>
       <c r="E12" s="42" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="F12" s="40" t="s">
         <v>70</v>
       </c>
       <c r="G12" s="53" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="H12" s="42" t="s">
         <v>71</v>
@@ -3769,7 +3766,7 @@
         <v>77</v>
       </c>
       <c r="G13" s="53" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="H13" s="42" t="s">
         <v>78</v>
@@ -3814,7 +3811,7 @@
         <v>82</v>
       </c>
       <c r="G14" s="53" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="H14" s="42" t="s">
         <v>83</v>
@@ -3859,7 +3856,7 @@
         <v>88</v>
       </c>
       <c r="G15" s="53" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="H15" s="42" t="s">
         <v>89</v>
@@ -3904,7 +3901,7 @@
         <v>93</v>
       </c>
       <c r="G16" s="53" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="H16" s="42" t="s">
         <v>94</v>
@@ -3949,7 +3946,7 @@
         <v>98</v>
       </c>
       <c r="G17" s="53" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="H17" s="42" t="s">
         <v>99</v>
@@ -3994,7 +3991,7 @@
         <v>104</v>
       </c>
       <c r="G18" s="53" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="H18" s="42" t="s">
         <v>105</v>
@@ -4036,13 +4033,13 @@
         <v>110</v>
       </c>
       <c r="F19" s="54" t="s">
+        <v>361</v>
+      </c>
+      <c r="G19" s="53" t="s">
         <v>362</v>
       </c>
-      <c r="G19" s="53" t="s">
-        <v>363</v>
-      </c>
       <c r="H19" s="48" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="I19" s="42"/>
       <c r="J19" s="38" t="s">
@@ -4052,7 +4049,7 @@
         <v>23</v>
       </c>
       <c r="L19" s="57" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="M19" s="38" t="s">
         <v>44</v>
@@ -4078,16 +4075,16 @@
         <v>18</v>
       </c>
       <c r="E20" s="55" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="F20" s="56" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="G20" s="53" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="H20" s="55" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="I20" s="44"/>
       <c r="J20" s="39" t="s">
@@ -4097,7 +4094,7 @@
         <v>23</v>
       </c>
       <c r="L20" s="57" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="M20" s="39" t="s">
         <v>44</v>
@@ -4217,7 +4214,7 @@
         <v>20</v>
       </c>
       <c r="G2" s="53" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="H2" s="42" t="s">
         <v>21</v>
@@ -4268,7 +4265,7 @@
         <v>29</v>
       </c>
       <c r="G3" s="53" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="H3" s="42" t="s">
         <v>30</v>
@@ -4319,7 +4316,7 @@
         <v>33</v>
       </c>
       <c r="G4" s="53" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="H4" s="42" t="s">
         <v>34</v>
@@ -4370,7 +4367,7 @@
         <v>38</v>
       </c>
       <c r="G5" s="53" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="H5" s="42" t="s">
         <v>39</v>
@@ -4421,7 +4418,7 @@
         <v>42</v>
       </c>
       <c r="G6" s="53" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="H6" s="42" t="s">
         <v>43</v>
@@ -4472,13 +4469,13 @@
         <v>47</v>
       </c>
       <c r="G7" s="53" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="H7" s="42" t="s">
         <v>48</v>
       </c>
       <c r="I7" s="48" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="J7" s="42"/>
       <c r="K7" s="38" t="s">
@@ -4497,7 +4494,7 @@
         <v>26</v>
       </c>
       <c r="P7" s="52" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="Q7" s="43" t="s">
         <v>23</v>
@@ -4523,7 +4520,7 @@
         <v>51</v>
       </c>
       <c r="G8" s="53" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="H8" s="42" t="s">
         <v>52</v>
@@ -4574,7 +4571,7 @@
         <v>55</v>
       </c>
       <c r="G9" s="53" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="H9" s="42" t="s">
         <v>56</v>
@@ -4625,7 +4622,7 @@
         <v>61</v>
       </c>
       <c r="G10" s="53" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="H10" s="42" t="s">
         <v>62</v>
@@ -4676,13 +4673,13 @@
         <v>66</v>
       </c>
       <c r="G11" s="53" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="H11" s="42" t="s">
         <v>67</v>
       </c>
       <c r="I11" s="48" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="J11" s="42"/>
       <c r="K11" s="38" t="s">
@@ -4701,7 +4698,7 @@
         <v>26</v>
       </c>
       <c r="P11" s="52" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="Q11" s="43" t="s">
         <v>23</v>
@@ -4721,19 +4718,19 @@
         <v>18</v>
       </c>
       <c r="E12" s="42" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="F12" s="40" t="s">
         <v>70</v>
       </c>
       <c r="G12" s="53" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="H12" s="42" t="s">
         <v>71</v>
       </c>
       <c r="I12" s="48" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="J12" s="42"/>
       <c r="K12" s="38" t="s">
@@ -4752,7 +4749,7 @@
         <v>26</v>
       </c>
       <c r="P12" s="52" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="Q12" s="43" t="s">
         <v>73</v>
@@ -4778,7 +4775,7 @@
         <v>77</v>
       </c>
       <c r="G13" s="53" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="H13" s="42" t="s">
         <v>78</v>
@@ -4829,7 +4826,7 @@
         <v>82</v>
       </c>
       <c r="G14" s="53" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="H14" s="42" t="s">
         <v>83</v>
@@ -4880,13 +4877,13 @@
         <v>88</v>
       </c>
       <c r="G15" s="53" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="H15" s="42" t="s">
         <v>89</v>
       </c>
       <c r="I15" s="48" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="J15" s="42"/>
       <c r="K15" s="38" t="s">
@@ -4905,7 +4902,7 @@
         <v>26</v>
       </c>
       <c r="P15" s="52" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="Q15" s="43" t="s">
         <v>23</v>
@@ -4931,7 +4928,7 @@
         <v>93</v>
       </c>
       <c r="G16" s="53" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="H16" s="42" t="s">
         <v>94</v>
@@ -4982,7 +4979,7 @@
         <v>98</v>
       </c>
       <c r="G17" s="53" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="H17" s="42" t="s">
         <v>99</v>
@@ -5033,7 +5030,7 @@
         <v>104</v>
       </c>
       <c r="G18" s="53" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="H18" s="42" t="s">
         <v>105</v>
@@ -5081,16 +5078,16 @@
         <v>110</v>
       </c>
       <c r="F19" s="54" t="s">
+        <v>361</v>
+      </c>
+      <c r="G19" s="53" t="s">
         <v>362</v>
       </c>
-      <c r="G19" s="53" t="s">
-        <v>363</v>
-      </c>
       <c r="H19" s="48" t="s">
+        <v>358</v>
+      </c>
+      <c r="I19" s="48" t="s">
         <v>359</v>
-      </c>
-      <c r="I19" s="48" t="s">
-        <v>360</v>
       </c>
       <c r="J19" s="42"/>
       <c r="K19" s="38" t="s">
@@ -5100,7 +5097,7 @@
         <v>23</v>
       </c>
       <c r="M19" s="57" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="N19" s="38" t="s">
         <v>44</v>
@@ -5109,7 +5106,7 @@
         <v>100</v>
       </c>
       <c r="P19" s="52" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="Q19" s="43" t="s">
         <v>23</v>
@@ -5129,19 +5126,19 @@
         <v>18</v>
       </c>
       <c r="E20" s="55" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="F20" s="56" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="G20" s="53" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="H20" s="55" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="I20" s="55" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="J20" s="44"/>
       <c r="K20" s="39" t="s">
@@ -5151,7 +5148,7 @@
         <v>23</v>
       </c>
       <c r="M20" s="57" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="N20" s="39" t="s">
         <v>44</v>
@@ -5160,7 +5157,7 @@
         <v>100</v>
       </c>
       <c r="P20" s="52" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="Q20" s="45" t="s">
         <v>23</v>

</xml_diff>